<commit_message>
feat(capa1): el MPI tambien se engancha al legajo por ID del Nino
Mismo criterio que el legajo y el MPE. `MPI 20260828 desproteg.xlsx`
identifica al chico solo por DNI y CUIL, asi que la nomina de proteccion
integral no se podia enganchar al legajo para los casos sin documento, que
son justamente los que mas lo necesitan.

Queda con las dos reglas: el ID tiene que existir en el legajo, y el CUIL
tiene que coincidir con el que el legajo declara para ese ID. La segunda
REUSA la definicion que ya usaba el MPE, aplicada a otro campo: es para
esto que la regla esta separada de su aplicacion.

De las tres nominas, ahora MPE y MPI se cruzan completas. El MPJ solo
verifica que el chico exista, porque su planilla no trae CUIL.

Las plantillas y los archivos de prueba de mir-v2 se regeneran: legajo,
MPE, MPI y MPJ traen el mismo ID y el mismo CUIL para la misma persona.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entorno/mir-v2/plantillas/MPI_2026_T1_MODELO.xlsx
+++ b/entorno/mir-v2/plantillas/MPI_2026_T1_MODELO.xlsx
@@ -114,8 +114,8 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -206,13 +206,21 @@
   <commentList>
     <comment ref="A3" authorId="0" shapeId="0">
       <text>
+        <t>ID del Niño, niña o Adolescente
+Identificador que le asigna el sistema provincial al niño, niña o adolescente. Es el mismo que figura en el legajo.
+Qué se espera: un número entero
+Campo obligatorio.</t>
+      </text>
+    </comment>
+    <comment ref="B3" authorId="0" shapeId="0">
+      <text>
         <t>Fecha del relevamiento
 Consignar la fecha en que se rrealiza el registro o actuliza la informacion.
 Qué se espera: una fecha, con formato dd/mm/aaaa
 Campo obligatorio.</t>
       </text>
     </comment>
-    <comment ref="B3" authorId="0" shapeId="0">
+    <comment ref="C3" authorId="0" shapeId="0">
       <text>
         <t>Provincia
 Qué se espera: texto
@@ -221,7 +229,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="C3" authorId="0" shapeId="0">
+    <comment ref="D3" authorId="0" shapeId="0">
       <text>
         <t>Nombre del programa/dispositivo
 Indicar el nombre del dispositivo, hogar, residencia, centro o programa donde se realiza la intervención.
@@ -230,7 +238,7 @@
 Campo obligatorio.</t>
       </text>
     </comment>
-    <comment ref="D3" authorId="0" shapeId="0">
+    <comment ref="E3" authorId="0" shapeId="0">
       <text>
         <t>Dependencia institucional
 Registrar la denominación oficial completa de la institución responsable, evitando siglas sin aclaración y nombres abreviados. Si el programa depende de más de un organismo, consignar la dependencia principal.
@@ -239,7 +247,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="E3" authorId="0" shapeId="0">
+    <comment ref="F3" authorId="0" shapeId="0">
       <text>
         <t>Localidad
 Qué se espera: texto
@@ -247,7 +255,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="F3" authorId="0" shapeId="0">
+    <comment ref="G3" authorId="0" shapeId="0">
       <text>
         <t>Domicilio
 Qué se espera: texto
@@ -255,7 +263,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="G3" authorId="0" shapeId="0">
+    <comment ref="H3" authorId="0" shapeId="0">
       <text>
         <t>Equipo interviniente
 Nombre del equipo o área interviniente. Profesionales que participan de la intervención (si corresponde). Disciplina o función de los integrantes cuando sea relevante.
@@ -264,7 +272,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="H3" authorId="0" shapeId="0">
+    <comment ref="I3" authorId="0" shapeId="0">
       <text>
         <t>Responsable del programa
 Nombre y apellido completos. Cargo o función (si corresponde). Persona formalmente designada como responsable del dispositivo o programa
@@ -273,7 +281,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="I3" authorId="0" shapeId="0">
+    <comment ref="J3" authorId="0" shapeId="0">
       <text>
         <t>Teléfono de contacto
 Qué se espera: texto
@@ -281,7 +289,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="J3" authorId="0" shapeId="0">
+    <comment ref="K3" authorId="0" shapeId="0">
       <text>
         <t>Mail de contacto
 Qué se espera: texto
@@ -289,7 +297,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="K3" authorId="0" shapeId="0">
+    <comment ref="L3" authorId="0" shapeId="0">
       <text>
         <t>Apellido/s
 Registrar el o los apellidos completos del niño, niña o adolescente, de acuerdo con la documentación vigente o, en su defecto, según la información proporcionada por la persona responsable o fuente institucional confiable
@@ -298,7 +306,7 @@
 Campo obligatorio.</t>
       </text>
     </comment>
-    <comment ref="L3" authorId="0" shapeId="0">
+    <comment ref="M3" authorId="0" shapeId="0">
       <text>
         <t>Nombre/s
 Registrar el o los nombres completos del niño, niña o adolescente, de acuerdo con la documentación vigente o, en su defecto, según la información proporcionada por la persona responsable o fuente institucional confiable
@@ -307,7 +315,7 @@
 Campo obligatorio.</t>
       </text>
     </comment>
-    <comment ref="M3" authorId="0" shapeId="0">
+    <comment ref="N3" authorId="0" shapeId="0">
       <text>
         <t>Situación de documentación
 Qué se espera: texto
@@ -316,7 +324,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="N3" authorId="0" shapeId="0">
+    <comment ref="O3" authorId="0" shapeId="0">
       <text>
         <t>Nº DNI
 Qué se espera: texto
@@ -324,7 +332,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="O3" authorId="0" shapeId="0">
+    <comment ref="P3" authorId="0" shapeId="0">
       <text>
         <t>Nº de CUIL
 Qué se espera: texto
@@ -332,7 +340,7 @@
 Campo obligatorio.</t>
       </text>
     </comment>
-    <comment ref="P3" authorId="0" shapeId="0">
+    <comment ref="Q3" authorId="0" shapeId="0">
       <text>
         <t>Género
 Qué se espera: texto
@@ -341,7 +349,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="Q3" authorId="0" shapeId="0">
+    <comment ref="R3" authorId="0" shapeId="0">
       <text>
         <t>País de nacimiento
 Qué se espera: texto
@@ -350,21 +358,21 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="R3" authorId="0" shapeId="0">
+    <comment ref="S3" authorId="0" shapeId="0">
       <text>
         <t>Fecha de nacimiento
 Qué se espera: una fecha, con formato dd/mm/aaaa
 Campo obligatorio.</t>
       </text>
     </comment>
-    <comment ref="S3" authorId="0" shapeId="0">
+    <comment ref="T3" authorId="0" shapeId="0">
       <text>
         <t>Edad
 Qué se espera: un número entero
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="T3" authorId="0" shapeId="0">
+    <comment ref="U3" authorId="0" shapeId="0">
       <text>
         <t>Asistencia escolar
 Qué se espera: texto
@@ -373,7 +381,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="U3" authorId="0" shapeId="0">
+    <comment ref="V3" authorId="0" shapeId="0">
       <text>
         <t>Máximo nivel educativo alcanzado
 Qué se espera: texto
@@ -382,7 +390,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="V3" authorId="0" shapeId="0">
+    <comment ref="W3" authorId="0" shapeId="0">
       <text>
         <t>Domicilio actual
 Qué se espera: texto
@@ -390,7 +398,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="W3" authorId="0" shapeId="0">
+    <comment ref="X3" authorId="0" shapeId="0">
       <text>
         <t>Provincia (NyA)
 Qué se espera: texto
@@ -399,7 +407,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="X3" authorId="0" shapeId="0">
+    <comment ref="Y3" authorId="0" shapeId="0">
       <text>
         <t>Localidad (NyA)
 Qué se espera: texto
@@ -407,7 +415,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="Y3" authorId="0" shapeId="0">
+    <comment ref="Z3" authorId="0" shapeId="0">
       <text>
         <t>Partido
 Qué se espera: texto
@@ -415,7 +423,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="Z3" authorId="0" shapeId="0">
+    <comment ref="AA3" authorId="0" shapeId="0">
       <text>
         <t>Código postal
 Qué se espera: texto
@@ -423,7 +431,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AA3" authorId="0" shapeId="0">
+    <comment ref="AB3" authorId="0" shapeId="0">
       <text>
         <t>Destinatario
 Consignar la persona, grupo poblacional o sujeto de derecho al que se dirige la intervención, prestación, acción de acompañamiento o medida de protección.
@@ -433,7 +441,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AB3" authorId="0" shapeId="0">
+    <comment ref="AC3" authorId="0" shapeId="0">
       <text>
         <t>Línea de acción
 Consignar la estrategia, componente programático, modalidad de intervención o eje de trabajo mediante el cual se implementa la acción de protección, promoción, restitución o fortalecimiento de derechos de NyA.
@@ -443,7 +451,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AC3" authorId="0" shapeId="0">
+    <comment ref="AD3" authorId="0" shapeId="0">
       <text>
         <t>Enfermedad crónica
 Registrar únicamente enfermedades crónicas diagnosticadas o informadas por fuentes confiables
@@ -452,7 +460,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AD3" authorId="0" shapeId="0">
+    <comment ref="AE3" authorId="0" shapeId="0">
       <text>
         <t>Problemática de salud
 Registrar cualquier situación, condición o dificultad vinculada a la salud física, mental o integral del Ny/Oa que requiera atención, seguimiento, tratamiento o articulación con servicios de salud, independientemente de que constituya o no una enfermedad crónica
@@ -462,7 +470,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AE3" authorId="0" shapeId="0">
+    <comment ref="AF3" authorId="0" shapeId="0">
       <text>
         <t>Consumo problemático de sustancias
 Registrar únicamente información conocida, relevada o informada por fuentes confiables. Cuando exista una situación de consumo, describirla de manera breve y objetiva
@@ -471,7 +479,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AF3" authorId="0" shapeId="0">
+    <comment ref="AG3" authorId="0" shapeId="0">
       <text>
         <t>¿Presenta alguna discapacidad?
 Qué se espera: texto
@@ -480,7 +488,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AG3" authorId="0" shapeId="0">
+    <comment ref="AH3" authorId="0" shapeId="0">
       <text>
         <t>Tipo de discapacidad
 Qué se espera: texto
@@ -489,7 +497,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AH3" authorId="0" shapeId="0">
+    <comment ref="AI3" authorId="0" shapeId="0">
       <text>
         <t>¿Posee CUD?
 Qué se espera: texto
@@ -498,7 +506,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AI3" authorId="0" shapeId="0">
+    <comment ref="AJ3" authorId="0" shapeId="0">
       <text>
         <t>Cobertura salud
 Qué se espera: texto
@@ -507,7 +515,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AJ3" authorId="0" shapeId="0">
+    <comment ref="AK3" authorId="0" shapeId="0">
       <text>
         <t>Seguridad social
 Registrar todos los beneficios vigentes. Ej:Asignación Universal por Hijo (AUH). Asignación Familiar. Pensión por discapacidad. Pensión no contributiva. Programa de acompañamiento social. Otro beneficio social
@@ -516,7 +524,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AK3" authorId="0" shapeId="0">
+    <comment ref="AL3" authorId="0" shapeId="0">
       <text>
         <t>¿Se identifica con algún pueblo originario?
 Identificar la pertenencia a pueblos originarios para contribuir a la producción de información con enfoque de derechos, diversidad cultural e interculturalidad
@@ -526,14 +534,14 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AL3" authorId="0" shapeId="0">
+    <comment ref="AM3" authorId="0" shapeId="0">
       <text>
         <t>Pueblo originario (especificar)
 Qué se espera: texto
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AM3" authorId="0" shapeId="0">
+    <comment ref="AN3" authorId="0" shapeId="0">
       <text>
         <t>¿Tiene hijos/as?
 Qué se espera: texto
@@ -542,7 +550,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AN3" authorId="0" shapeId="0">
+    <comment ref="AO3" authorId="0" shapeId="0">
       <text>
         <t>Relación vincular del referente
 Qué se espera: texto
@@ -551,7 +559,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AO3" authorId="0" shapeId="0">
+    <comment ref="AP3" authorId="0" shapeId="0">
       <text>
         <t>Apellido/s del referente
 Qué se espera: texto
@@ -559,7 +567,7 @@
 Campo obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AP3" authorId="0" shapeId="0">
+    <comment ref="AQ3" authorId="0" shapeId="0">
       <text>
         <t>Nombre/s del referente
 Qué se espera: texto
@@ -567,7 +575,7 @@
 Campo obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AQ3" authorId="0" shapeId="0">
+    <comment ref="AR3" authorId="0" shapeId="0">
       <text>
         <t>DNI del referente
 Qué se espera: texto
@@ -575,7 +583,7 @@
 Campo obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AR3" authorId="0" shapeId="0">
+    <comment ref="AS3" authorId="0" shapeId="0">
       <text>
         <t>Género del referente
 Qué se espera: texto
@@ -584,14 +592,14 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AS3" authorId="0" shapeId="0">
+    <comment ref="AT3" authorId="0" shapeId="0">
       <text>
         <t>Fecha de nacimiento del referente
 Qué se espera: una fecha, con formato dd/mm/aaaa
 Campo obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AT3" authorId="0" shapeId="0">
+    <comment ref="AU3" authorId="0" shapeId="0">
       <text>
         <t>Nacionalidad del referente
 Qué se espera: texto
@@ -600,7 +608,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AU3" authorId="0" shapeId="0">
+    <comment ref="AV3" authorId="0" shapeId="0">
       <text>
         <t>Domicilio actual del referente
 Qué se espera: texto
@@ -608,7 +616,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AV3" authorId="0" shapeId="0">
+    <comment ref="AW3" authorId="0" shapeId="0">
       <text>
         <t>Código postal del referente
 Qué se espera: texto
@@ -616,7 +624,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AW3" authorId="0" shapeId="0">
+    <comment ref="AX3" authorId="0" shapeId="0">
       <text>
         <t>Localidad del referente
 Qué se espera: texto
@@ -624,7 +632,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AX3" authorId="0" shapeId="0">
+    <comment ref="AY3" authorId="0" shapeId="0">
       <text>
         <t>Partido del referente
 Qué se espera: texto
@@ -632,7 +640,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AY3" authorId="0" shapeId="0">
+    <comment ref="AZ3" authorId="0" shapeId="0">
       <text>
         <t>Provincia del referente
 Qué se espera: texto
@@ -641,7 +649,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="AZ3" authorId="0" shapeId="0">
+    <comment ref="BA3" authorId="0" shapeId="0">
       <text>
         <t>Teléfono y mail del referente
 Qué se espera: texto
@@ -649,7 +657,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BA3" authorId="0" shapeId="0">
+    <comment ref="BB3" authorId="0" shapeId="0">
       <text>
         <t>Nivel escolar del referente
 Qué se espera: texto
@@ -658,7 +666,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BB3" authorId="0" shapeId="0">
+    <comment ref="BC3" authorId="0" shapeId="0">
       <text>
         <t>Situación laboral del referente
 Qué se espera: texto
@@ -667,7 +675,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BC3" authorId="0" shapeId="0">
+    <comment ref="BD3" authorId="0" shapeId="0">
       <text>
         <t>Seguridad social del referente
 Qué se espera: texto
@@ -675,7 +683,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BD3" authorId="0" shapeId="0">
+    <comment ref="BE3" authorId="0" shapeId="0">
       <text>
         <t>¿El referente se identifica con algún pueblo originario?
 Qué se espera: texto
@@ -684,7 +692,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BE3" authorId="0" shapeId="0">
+    <comment ref="BF3" authorId="0" shapeId="0">
       <text>
         <t>Pueblo originario del refrente
 Qué se espera: texto
@@ -692,7 +700,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BF3" authorId="0" shapeId="0">
+    <comment ref="BG3" authorId="0" shapeId="0">
       <text>
         <t>Equipo Interviniente
 Debe identificarse prioritariamente el equipo, área o servicio de pertenencia. Si intervienen varios equipos, consignar el que tenga la responsabilidad principal de la medida o coordinación del caso.
@@ -701,7 +709,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BG3" authorId="0" shapeId="0">
+    <comment ref="BH3" authorId="0" shapeId="0">
       <text>
         <t>Origen de la demanda
 Qué se espera: texto
@@ -710,7 +718,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BH3" authorId="0" shapeId="0">
+    <comment ref="BI3" authorId="0" shapeId="0">
       <text>
         <t>Causas de las medidas
 Mencionar la causa principal que motivó la implementación de la medida. Cuando existan múltiples situaciones de vulneración, registrar aquella que resulte predominante o que haya dado origen a la intervención.
@@ -719,7 +727,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BI3" authorId="0" shapeId="0">
+    <comment ref="BJ3" authorId="0" shapeId="0">
       <text>
         <t>Fecha de la medida MPI
 Registrar la fecha en que se dictó, dispuso o formalizó la Medida de Protección Integral (MPI) por parte de la autoridad administrativa competente. Esta fecha marca el inicio formal de la intervención en el marco de la medida
@@ -727,7 +735,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BJ3" authorId="0" shapeId="0">
+    <comment ref="BK3" authorId="0" shapeId="0">
       <text>
         <t>Plazos en la intervención
 Consignar el período previsto o establecido para la implementación, seguimiento y evaluación de la Medida de Protección Integral (MPI), de acuerdo con la planificación realizada por el organismo o equipo interviniente.
@@ -736,7 +744,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BK3" authorId="0" shapeId="0">
+    <comment ref="BL3" authorId="0" shapeId="0">
       <text>
         <t>Causas del cese de la MPI
 Identificar los motivos de finalización de las Medidas de Protección Integral y contribuir al monitoreo de los resultados alcanzados en los procesos de restitución y garantía de derechos
@@ -745,7 +753,7 @@
 No es obligatorio.</t>
       </text>
     </comment>
-    <comment ref="BL3" authorId="0" shapeId="0">
+    <comment ref="BM3" authorId="0" shapeId="0">
       <text>
         <t>Observaciones
 Registrar información complementaria relevante que contribuya a una mejor comprensión de la situación del niño, niña o adolescente, de su contexto familiar o de la intervención realizada, y que no haya sido consignada en otros campos del formulario.
@@ -1046,73 +1054,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL203"/>
+  <dimension ref="A1:BM203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
     <col width="17" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="24" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
     <col width="15" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="14" customWidth="1" min="27" max="27"/>
-    <col width="15" customWidth="1" min="28" max="28"/>
-    <col width="17" customWidth="1" min="29" max="29"/>
-    <col width="18" customWidth="1" min="30" max="30"/>
-    <col width="25" customWidth="1" min="31" max="31"/>
-    <col width="23" customWidth="1" min="32" max="32"/>
-    <col width="18" customWidth="1" min="33" max="33"/>
-    <col width="14" customWidth="1" min="34" max="34"/>
-    <col width="15" customWidth="1" min="35" max="35"/>
-    <col width="16" customWidth="1" min="36" max="36"/>
-    <col width="29" customWidth="1" min="37" max="37"/>
-    <col width="23" customWidth="1" min="38" max="38"/>
-    <col width="16" customWidth="1" min="39" max="39"/>
-    <col width="23" customWidth="1" min="40" max="40"/>
-    <col width="20" customWidth="1" min="41" max="41"/>
-    <col width="19" customWidth="1" min="42" max="42"/>
-    <col width="16" customWidth="1" min="43" max="43"/>
-    <col width="18" customWidth="1" min="44" max="44"/>
-    <col width="24" customWidth="1" min="45" max="45"/>
-    <col width="21" customWidth="1" min="46" max="46"/>
-    <col width="23" customWidth="1" min="47" max="47"/>
-    <col width="21" customWidth="1" min="48" max="48"/>
-    <col width="19" customWidth="1" min="49" max="49"/>
-    <col width="18" customWidth="1" min="50" max="50"/>
-    <col width="19" customWidth="1" min="51" max="51"/>
-    <col width="22" customWidth="1" min="52" max="52"/>
-    <col width="21" customWidth="1" min="53" max="53"/>
-    <col width="23" customWidth="1" min="54" max="54"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="15" customWidth="1" min="29" max="29"/>
+    <col width="17" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="25" customWidth="1" min="32" max="32"/>
+    <col width="23" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="14" customWidth="1" min="35" max="35"/>
+    <col width="15" customWidth="1" min="36" max="36"/>
+    <col width="16" customWidth="1" min="37" max="37"/>
+    <col width="29" customWidth="1" min="38" max="38"/>
+    <col width="23" customWidth="1" min="39" max="39"/>
+    <col width="16" customWidth="1" min="40" max="40"/>
+    <col width="23" customWidth="1" min="41" max="41"/>
+    <col width="20" customWidth="1" min="42" max="42"/>
+    <col width="19" customWidth="1" min="43" max="43"/>
+    <col width="16" customWidth="1" min="44" max="44"/>
+    <col width="18" customWidth="1" min="45" max="45"/>
+    <col width="24" customWidth="1" min="46" max="46"/>
+    <col width="21" customWidth="1" min="47" max="47"/>
+    <col width="23" customWidth="1" min="48" max="48"/>
+    <col width="21" customWidth="1" min="49" max="49"/>
+    <col width="19" customWidth="1" min="50" max="50"/>
+    <col width="18" customWidth="1" min="51" max="51"/>
+    <col width="19" customWidth="1" min="52" max="52"/>
+    <col width="22" customWidth="1" min="53" max="53"/>
+    <col width="21" customWidth="1" min="54" max="54"/>
     <col width="23" customWidth="1" min="55" max="55"/>
-    <col width="36" customWidth="1" min="56" max="56"/>
-    <col width="23" customWidth="1" min="57" max="57"/>
-    <col width="18" customWidth="1" min="58" max="58"/>
+    <col width="23" customWidth="1" min="56" max="56"/>
+    <col width="36" customWidth="1" min="57" max="57"/>
+    <col width="23" customWidth="1" min="58" max="58"/>
     <col width="18" customWidth="1" min="59" max="59"/>
     <col width="18" customWidth="1" min="60" max="60"/>
-    <col width="19" customWidth="1" min="61" max="61"/>
-    <col width="20" customWidth="1" min="62" max="62"/>
+    <col width="18" customWidth="1" min="61" max="61"/>
+    <col width="19" customWidth="1" min="62" max="62"/>
     <col width="20" customWidth="1" min="63" max="63"/>
-    <col width="14" customWidth="1" min="64" max="64"/>
+    <col width="20" customWidth="1" min="64" max="64"/>
+    <col width="14" customWidth="1" min="65" max="65"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1123,22 +1132,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Dispositivo/espacio</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Niño o adolescente</t>
         </is>
       </c>
-      <c r="AN2" s="2" t="inlineStr">
+      <c r="AO2" s="2" t="inlineStr">
         <is>
           <t>Referente</t>
         </is>
       </c>
-      <c r="BF2" s="2" t="inlineStr">
+      <c r="BG2" s="2" t="inlineStr">
         <is>
           <t>Medida</t>
         </is>
@@ -1147,320 +1156,325 @@
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
+          <t>ID del Niño, niña o Adolescente *</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
           <t>Fecha del relevamiento *</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Provincia</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Nombre del programa/dispositivo *</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Dependencia institucional</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Localidad</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Domicilio</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>Equipo interviniente</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Responsable del programa</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Teléfono de contacto</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Mail de contacto</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Apellido/s *</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Nombre/s *</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Situación de documentación</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>Nº DNI</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Nº de CUIL *</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="Q3" s="4" t="inlineStr">
         <is>
           <t>Género</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="R3" s="4" t="inlineStr">
         <is>
           <t>País de nacimiento</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>Fecha de nacimiento *</t>
         </is>
       </c>
-      <c r="S3" s="4" t="inlineStr">
+      <c r="T3" s="4" t="inlineStr">
         <is>
           <t>Edad</t>
         </is>
       </c>
-      <c r="T3" s="4" t="inlineStr">
+      <c r="U3" s="4" t="inlineStr">
         <is>
           <t>Asistencia escolar</t>
         </is>
       </c>
-      <c r="U3" s="4" t="inlineStr">
+      <c r="V3" s="4" t="inlineStr">
         <is>
           <t>Máximo nivel educativo alcanzado</t>
         </is>
       </c>
-      <c r="V3" s="4" t="inlineStr">
+      <c r="W3" s="4" t="inlineStr">
         <is>
           <t>Domicilio actual</t>
         </is>
       </c>
-      <c r="W3" s="4" t="inlineStr">
+      <c r="X3" s="4" t="inlineStr">
         <is>
           <t>Provincia (NyA)</t>
         </is>
       </c>
-      <c r="X3" s="4" t="inlineStr">
+      <c r="Y3" s="4" t="inlineStr">
         <is>
           <t>Localidad (NyA)</t>
         </is>
       </c>
-      <c r="Y3" s="4" t="inlineStr">
+      <c r="Z3" s="4" t="inlineStr">
         <is>
           <t>Partido</t>
         </is>
       </c>
-      <c r="Z3" s="4" t="inlineStr">
+      <c r="AA3" s="4" t="inlineStr">
         <is>
           <t>Código postal</t>
         </is>
       </c>
-      <c r="AA3" s="4" t="inlineStr">
+      <c r="AB3" s="4" t="inlineStr">
         <is>
           <t>Destinatario</t>
         </is>
       </c>
-      <c r="AB3" s="4" t="inlineStr">
+      <c r="AC3" s="4" t="inlineStr">
         <is>
           <t>Línea de acción</t>
         </is>
       </c>
-      <c r="AC3" s="4" t="inlineStr">
+      <c r="AD3" s="4" t="inlineStr">
         <is>
           <t>Enfermedad crónica</t>
         </is>
       </c>
-      <c r="AD3" s="4" t="inlineStr">
+      <c r="AE3" s="4" t="inlineStr">
         <is>
           <t>Problemática de salud</t>
         </is>
       </c>
-      <c r="AE3" s="4" t="inlineStr">
+      <c r="AF3" s="4" t="inlineStr">
         <is>
           <t>Consumo problemático de sustancias</t>
         </is>
       </c>
-      <c r="AF3" s="4" t="inlineStr">
+      <c r="AG3" s="4" t="inlineStr">
         <is>
           <t>¿Presenta alguna discapacidad?</t>
         </is>
       </c>
-      <c r="AG3" s="4" t="inlineStr">
+      <c r="AH3" s="4" t="inlineStr">
         <is>
           <t>Tipo de discapacidad</t>
         </is>
       </c>
-      <c r="AH3" s="4" t="inlineStr">
+      <c r="AI3" s="4" t="inlineStr">
         <is>
           <t>¿Posee CUD?</t>
         </is>
       </c>
-      <c r="AI3" s="4" t="inlineStr">
+      <c r="AJ3" s="4" t="inlineStr">
         <is>
           <t>Cobertura salud</t>
         </is>
       </c>
-      <c r="AJ3" s="4" t="inlineStr">
+      <c r="AK3" s="4" t="inlineStr">
         <is>
           <t>Seguridad social</t>
         </is>
       </c>
-      <c r="AK3" s="4" t="inlineStr">
+      <c r="AL3" s="4" t="inlineStr">
         <is>
           <t>¿Se identifica con algún pueblo originario?</t>
         </is>
       </c>
-      <c r="AL3" s="4" t="inlineStr">
+      <c r="AM3" s="4" t="inlineStr">
         <is>
           <t>Pueblo originario (especificar)</t>
         </is>
       </c>
-      <c r="AM3" s="4" t="inlineStr">
+      <c r="AN3" s="4" t="inlineStr">
         <is>
           <t>¿Tiene hijos/as?</t>
         </is>
       </c>
-      <c r="AN3" s="4" t="inlineStr">
+      <c r="AO3" s="4" t="inlineStr">
         <is>
           <t>Relación vincular del referente</t>
         </is>
       </c>
-      <c r="AO3" s="3" t="inlineStr">
+      <c r="AP3" s="3" t="inlineStr">
         <is>
           <t>Apellido/s del referente *</t>
         </is>
       </c>
-      <c r="AP3" s="3" t="inlineStr">
+      <c r="AQ3" s="3" t="inlineStr">
         <is>
           <t>Nombre/s del referente *</t>
         </is>
       </c>
-      <c r="AQ3" s="3" t="inlineStr">
+      <c r="AR3" s="3" t="inlineStr">
         <is>
           <t>DNI del referente *</t>
         </is>
       </c>
-      <c r="AR3" s="4" t="inlineStr">
+      <c r="AS3" s="4" t="inlineStr">
         <is>
           <t>Género del referente</t>
         </is>
       </c>
-      <c r="AS3" s="3" t="inlineStr">
+      <c r="AT3" s="3" t="inlineStr">
         <is>
           <t>Fecha de nacimiento del referente *</t>
         </is>
       </c>
-      <c r="AT3" s="4" t="inlineStr">
+      <c r="AU3" s="4" t="inlineStr">
         <is>
           <t>Nacionalidad del referente</t>
         </is>
       </c>
-      <c r="AU3" s="4" t="inlineStr">
+      <c r="AV3" s="4" t="inlineStr">
         <is>
           <t>Domicilio actual del referente</t>
         </is>
       </c>
-      <c r="AV3" s="4" t="inlineStr">
+      <c r="AW3" s="4" t="inlineStr">
         <is>
           <t>Código postal del referente</t>
         </is>
       </c>
-      <c r="AW3" s="4" t="inlineStr">
+      <c r="AX3" s="4" t="inlineStr">
         <is>
           <t>Localidad del referente</t>
         </is>
       </c>
-      <c r="AX3" s="4" t="inlineStr">
+      <c r="AY3" s="4" t="inlineStr">
         <is>
           <t>Partido del referente</t>
         </is>
       </c>
-      <c r="AY3" s="4" t="inlineStr">
+      <c r="AZ3" s="4" t="inlineStr">
         <is>
           <t>Provincia del referente</t>
         </is>
       </c>
-      <c r="AZ3" s="4" t="inlineStr">
+      <c r="BA3" s="4" t="inlineStr">
         <is>
           <t>Teléfono y mail del referente</t>
         </is>
       </c>
-      <c r="BA3" s="4" t="inlineStr">
+      <c r="BB3" s="4" t="inlineStr">
         <is>
           <t>Nivel escolar del referente</t>
         </is>
       </c>
-      <c r="BB3" s="4" t="inlineStr">
+      <c r="BC3" s="4" t="inlineStr">
         <is>
           <t>Situación laboral del referente</t>
         </is>
       </c>
-      <c r="BC3" s="4" t="inlineStr">
+      <c r="BD3" s="4" t="inlineStr">
         <is>
           <t>Seguridad social del referente</t>
         </is>
       </c>
-      <c r="BD3" s="4" t="inlineStr">
+      <c r="BE3" s="4" t="inlineStr">
         <is>
           <t>¿El referente se identifica con algún pueblo originario?</t>
         </is>
       </c>
-      <c r="BE3" s="4" t="inlineStr">
+      <c r="BF3" s="4" t="inlineStr">
         <is>
           <t>Pueblo originario del refrente</t>
         </is>
       </c>
-      <c r="BF3" s="4" t="inlineStr">
+      <c r="BG3" s="4" t="inlineStr">
         <is>
           <t>Equipo Interviniente</t>
         </is>
       </c>
-      <c r="BG3" s="4" t="inlineStr">
+      <c r="BH3" s="4" t="inlineStr">
         <is>
           <t>Origen de la demanda</t>
         </is>
       </c>
-      <c r="BH3" s="4" t="inlineStr">
+      <c r="BI3" s="4" t="inlineStr">
         <is>
           <t>Causas de las medidas</t>
         </is>
       </c>
-      <c r="BI3" s="4" t="inlineStr">
+      <c r="BJ3" s="4" t="inlineStr">
         <is>
           <t>Fecha de la medida MPI</t>
         </is>
       </c>
-      <c r="BJ3" s="4" t="inlineStr">
+      <c r="BK3" s="4" t="inlineStr">
         <is>
           <t>Plazos en la intervención</t>
         </is>
       </c>
-      <c r="BK3" s="4" t="inlineStr">
+      <c r="BL3" s="4" t="inlineStr">
         <is>
           <t>Causas del cese de la MPI</t>
         </is>
       </c>
-      <c r="BL3" s="4" t="inlineStr">
+      <c r="BM3" s="4" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1468,1483 +1482,1683 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n"/>
-      <c r="R4" s="5" t="n"/>
+      <c r="B4" s="6" t="n"/>
       <c r="S4" s="6" t="n"/>
-      <c r="AS4" s="5" t="n"/>
-      <c r="BI4" s="5" t="n"/>
+      <c r="T4" s="5" t="n"/>
+      <c r="AT4" s="6" t="n"/>
+      <c r="BJ4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
-      <c r="R5" s="5" t="n"/>
+      <c r="B5" s="6" t="n"/>
       <c r="S5" s="6" t="n"/>
-      <c r="AS5" s="5" t="n"/>
-      <c r="BI5" s="5" t="n"/>
+      <c r="T5" s="5" t="n"/>
+      <c r="AT5" s="6" t="n"/>
+      <c r="BJ5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
+      <c r="B6" s="6" t="n"/>
       <c r="S6" s="6" t="n"/>
-      <c r="AS6" s="5" t="n"/>
-      <c r="BI6" s="5" t="n"/>
+      <c r="T6" s="5" t="n"/>
+      <c r="AT6" s="6" t="n"/>
+      <c r="BJ6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
-      <c r="R7" s="5" t="n"/>
+      <c r="B7" s="6" t="n"/>
       <c r="S7" s="6" t="n"/>
-      <c r="AS7" s="5" t="n"/>
-      <c r="BI7" s="5" t="n"/>
+      <c r="T7" s="5" t="n"/>
+      <c r="AT7" s="6" t="n"/>
+      <c r="BJ7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
-      <c r="R8" s="5" t="n"/>
+      <c r="B8" s="6" t="n"/>
       <c r="S8" s="6" t="n"/>
-      <c r="AS8" s="5" t="n"/>
-      <c r="BI8" s="5" t="n"/>
+      <c r="T8" s="5" t="n"/>
+      <c r="AT8" s="6" t="n"/>
+      <c r="BJ8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
-      <c r="R9" s="5" t="n"/>
+      <c r="B9" s="6" t="n"/>
       <c r="S9" s="6" t="n"/>
-      <c r="AS9" s="5" t="n"/>
-      <c r="BI9" s="5" t="n"/>
+      <c r="T9" s="5" t="n"/>
+      <c r="AT9" s="6" t="n"/>
+      <c r="BJ9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
-      <c r="R10" s="5" t="n"/>
+      <c r="B10" s="6" t="n"/>
       <c r="S10" s="6" t="n"/>
-      <c r="AS10" s="5" t="n"/>
-      <c r="BI10" s="5" t="n"/>
+      <c r="T10" s="5" t="n"/>
+      <c r="AT10" s="6" t="n"/>
+      <c r="BJ10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
-      <c r="R11" s="5" t="n"/>
+      <c r="B11" s="6" t="n"/>
       <c r="S11" s="6" t="n"/>
-      <c r="AS11" s="5" t="n"/>
-      <c r="BI11" s="5" t="n"/>
+      <c r="T11" s="5" t="n"/>
+      <c r="AT11" s="6" t="n"/>
+      <c r="BJ11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
-      <c r="R12" s="5" t="n"/>
+      <c r="B12" s="6" t="n"/>
       <c r="S12" s="6" t="n"/>
-      <c r="AS12" s="5" t="n"/>
-      <c r="BI12" s="5" t="n"/>
+      <c r="T12" s="5" t="n"/>
+      <c r="AT12" s="6" t="n"/>
+      <c r="BJ12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
-      <c r="R13" s="5" t="n"/>
+      <c r="B13" s="6" t="n"/>
       <c r="S13" s="6" t="n"/>
-      <c r="AS13" s="5" t="n"/>
-      <c r="BI13" s="5" t="n"/>
+      <c r="T13" s="5" t="n"/>
+      <c r="AT13" s="6" t="n"/>
+      <c r="BJ13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
-      <c r="R14" s="5" t="n"/>
+      <c r="B14" s="6" t="n"/>
       <c r="S14" s="6" t="n"/>
-      <c r="AS14" s="5" t="n"/>
-      <c r="BI14" s="5" t="n"/>
+      <c r="T14" s="5" t="n"/>
+      <c r="AT14" s="6" t="n"/>
+      <c r="BJ14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
-      <c r="R15" s="5" t="n"/>
+      <c r="B15" s="6" t="n"/>
       <c r="S15" s="6" t="n"/>
-      <c r="AS15" s="5" t="n"/>
-      <c r="BI15" s="5" t="n"/>
+      <c r="T15" s="5" t="n"/>
+      <c r="AT15" s="6" t="n"/>
+      <c r="BJ15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
-      <c r="R16" s="5" t="n"/>
+      <c r="B16" s="6" t="n"/>
       <c r="S16" s="6" t="n"/>
-      <c r="AS16" s="5" t="n"/>
-      <c r="BI16" s="5" t="n"/>
+      <c r="T16" s="5" t="n"/>
+      <c r="AT16" s="6" t="n"/>
+      <c r="BJ16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
-      <c r="R17" s="5" t="n"/>
+      <c r="B17" s="6" t="n"/>
       <c r="S17" s="6" t="n"/>
-      <c r="AS17" s="5" t="n"/>
-      <c r="BI17" s="5" t="n"/>
+      <c r="T17" s="5" t="n"/>
+      <c r="AT17" s="6" t="n"/>
+      <c r="BJ17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
-      <c r="R18" s="5" t="n"/>
+      <c r="B18" s="6" t="n"/>
       <c r="S18" s="6" t="n"/>
-      <c r="AS18" s="5" t="n"/>
-      <c r="BI18" s="5" t="n"/>
+      <c r="T18" s="5" t="n"/>
+      <c r="AT18" s="6" t="n"/>
+      <c r="BJ18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
-      <c r="R19" s="5" t="n"/>
+      <c r="B19" s="6" t="n"/>
       <c r="S19" s="6" t="n"/>
-      <c r="AS19" s="5" t="n"/>
-      <c r="BI19" s="5" t="n"/>
+      <c r="T19" s="5" t="n"/>
+      <c r="AT19" s="6" t="n"/>
+      <c r="BJ19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n"/>
-      <c r="R20" s="5" t="n"/>
+      <c r="B20" s="6" t="n"/>
       <c r="S20" s="6" t="n"/>
-      <c r="AS20" s="5" t="n"/>
-      <c r="BI20" s="5" t="n"/>
+      <c r="T20" s="5" t="n"/>
+      <c r="AT20" s="6" t="n"/>
+      <c r="BJ20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
-      <c r="R21" s="5" t="n"/>
+      <c r="B21" s="6" t="n"/>
       <c r="S21" s="6" t="n"/>
-      <c r="AS21" s="5" t="n"/>
-      <c r="BI21" s="5" t="n"/>
+      <c r="T21" s="5" t="n"/>
+      <c r="AT21" s="6" t="n"/>
+      <c r="BJ21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
-      <c r="R22" s="5" t="n"/>
+      <c r="B22" s="6" t="n"/>
       <c r="S22" s="6" t="n"/>
-      <c r="AS22" s="5" t="n"/>
-      <c r="BI22" s="5" t="n"/>
+      <c r="T22" s="5" t="n"/>
+      <c r="AT22" s="6" t="n"/>
+      <c r="BJ22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
-      <c r="R23" s="5" t="n"/>
+      <c r="B23" s="6" t="n"/>
       <c r="S23" s="6" t="n"/>
-      <c r="AS23" s="5" t="n"/>
-      <c r="BI23" s="5" t="n"/>
+      <c r="T23" s="5" t="n"/>
+      <c r="AT23" s="6" t="n"/>
+      <c r="BJ23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n"/>
-      <c r="R24" s="5" t="n"/>
+      <c r="B24" s="6" t="n"/>
       <c r="S24" s="6" t="n"/>
-      <c r="AS24" s="5" t="n"/>
-      <c r="BI24" s="5" t="n"/>
+      <c r="T24" s="5" t="n"/>
+      <c r="AT24" s="6" t="n"/>
+      <c r="BJ24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
-      <c r="R25" s="5" t="n"/>
+      <c r="B25" s="6" t="n"/>
       <c r="S25" s="6" t="n"/>
-      <c r="AS25" s="5" t="n"/>
-      <c r="BI25" s="5" t="n"/>
+      <c r="T25" s="5" t="n"/>
+      <c r="AT25" s="6" t="n"/>
+      <c r="BJ25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n"/>
-      <c r="R26" s="5" t="n"/>
+      <c r="B26" s="6" t="n"/>
       <c r="S26" s="6" t="n"/>
-      <c r="AS26" s="5" t="n"/>
-      <c r="BI26" s="5" t="n"/>
+      <c r="T26" s="5" t="n"/>
+      <c r="AT26" s="6" t="n"/>
+      <c r="BJ26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
-      <c r="R27" s="5" t="n"/>
+      <c r="B27" s="6" t="n"/>
       <c r="S27" s="6" t="n"/>
-      <c r="AS27" s="5" t="n"/>
-      <c r="BI27" s="5" t="n"/>
+      <c r="T27" s="5" t="n"/>
+      <c r="AT27" s="6" t="n"/>
+      <c r="BJ27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n"/>
-      <c r="R28" s="5" t="n"/>
+      <c r="B28" s="6" t="n"/>
       <c r="S28" s="6" t="n"/>
-      <c r="AS28" s="5" t="n"/>
-      <c r="BI28" s="5" t="n"/>
+      <c r="T28" s="5" t="n"/>
+      <c r="AT28" s="6" t="n"/>
+      <c r="BJ28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
-      <c r="R29" s="5" t="n"/>
+      <c r="B29" s="6" t="n"/>
       <c r="S29" s="6" t="n"/>
-      <c r="AS29" s="5" t="n"/>
-      <c r="BI29" s="5" t="n"/>
+      <c r="T29" s="5" t="n"/>
+      <c r="AT29" s="6" t="n"/>
+      <c r="BJ29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n"/>
-      <c r="R30" s="5" t="n"/>
+      <c r="B30" s="6" t="n"/>
       <c r="S30" s="6" t="n"/>
-      <c r="AS30" s="5" t="n"/>
-      <c r="BI30" s="5" t="n"/>
+      <c r="T30" s="5" t="n"/>
+      <c r="AT30" s="6" t="n"/>
+      <c r="BJ30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
-      <c r="R31" s="5" t="n"/>
+      <c r="B31" s="6" t="n"/>
       <c r="S31" s="6" t="n"/>
-      <c r="AS31" s="5" t="n"/>
-      <c r="BI31" s="5" t="n"/>
+      <c r="T31" s="5" t="n"/>
+      <c r="AT31" s="6" t="n"/>
+      <c r="BJ31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>
-      <c r="R32" s="5" t="n"/>
+      <c r="B32" s="6" t="n"/>
       <c r="S32" s="6" t="n"/>
-      <c r="AS32" s="5" t="n"/>
-      <c r="BI32" s="5" t="n"/>
+      <c r="T32" s="5" t="n"/>
+      <c r="AT32" s="6" t="n"/>
+      <c r="BJ32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n"/>
-      <c r="R33" s="5" t="n"/>
+      <c r="B33" s="6" t="n"/>
       <c r="S33" s="6" t="n"/>
-      <c r="AS33" s="5" t="n"/>
-      <c r="BI33" s="5" t="n"/>
+      <c r="T33" s="5" t="n"/>
+      <c r="AT33" s="6" t="n"/>
+      <c r="BJ33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n"/>
-      <c r="R34" s="5" t="n"/>
+      <c r="B34" s="6" t="n"/>
       <c r="S34" s="6" t="n"/>
-      <c r="AS34" s="5" t="n"/>
-      <c r="BI34" s="5" t="n"/>
+      <c r="T34" s="5" t="n"/>
+      <c r="AT34" s="6" t="n"/>
+      <c r="BJ34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n"/>
-      <c r="R35" s="5" t="n"/>
+      <c r="B35" s="6" t="n"/>
       <c r="S35" s="6" t="n"/>
-      <c r="AS35" s="5" t="n"/>
-      <c r="BI35" s="5" t="n"/>
+      <c r="T35" s="5" t="n"/>
+      <c r="AT35" s="6" t="n"/>
+      <c r="BJ35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n"/>
-      <c r="R36" s="5" t="n"/>
+      <c r="B36" s="6" t="n"/>
       <c r="S36" s="6" t="n"/>
-      <c r="AS36" s="5" t="n"/>
-      <c r="BI36" s="5" t="n"/>
+      <c r="T36" s="5" t="n"/>
+      <c r="AT36" s="6" t="n"/>
+      <c r="BJ36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
-      <c r="R37" s="5" t="n"/>
+      <c r="B37" s="6" t="n"/>
       <c r="S37" s="6" t="n"/>
-      <c r="AS37" s="5" t="n"/>
-      <c r="BI37" s="5" t="n"/>
+      <c r="T37" s="5" t="n"/>
+      <c r="AT37" s="6" t="n"/>
+      <c r="BJ37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n"/>
-      <c r="R38" s="5" t="n"/>
+      <c r="B38" s="6" t="n"/>
       <c r="S38" s="6" t="n"/>
-      <c r="AS38" s="5" t="n"/>
-      <c r="BI38" s="5" t="n"/>
+      <c r="T38" s="5" t="n"/>
+      <c r="AT38" s="6" t="n"/>
+      <c r="BJ38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
-      <c r="R39" s="5" t="n"/>
+      <c r="B39" s="6" t="n"/>
       <c r="S39" s="6" t="n"/>
-      <c r="AS39" s="5" t="n"/>
-      <c r="BI39" s="5" t="n"/>
+      <c r="T39" s="5" t="n"/>
+      <c r="AT39" s="6" t="n"/>
+      <c r="BJ39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n"/>
-      <c r="R40" s="5" t="n"/>
+      <c r="B40" s="6" t="n"/>
       <c r="S40" s="6" t="n"/>
-      <c r="AS40" s="5" t="n"/>
-      <c r="BI40" s="5" t="n"/>
+      <c r="T40" s="5" t="n"/>
+      <c r="AT40" s="6" t="n"/>
+      <c r="BJ40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
-      <c r="R41" s="5" t="n"/>
+      <c r="B41" s="6" t="n"/>
       <c r="S41" s="6" t="n"/>
-      <c r="AS41" s="5" t="n"/>
-      <c r="BI41" s="5" t="n"/>
+      <c r="T41" s="5" t="n"/>
+      <c r="AT41" s="6" t="n"/>
+      <c r="BJ41" s="6" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n"/>
-      <c r="R42" s="5" t="n"/>
+      <c r="B42" s="6" t="n"/>
       <c r="S42" s="6" t="n"/>
-      <c r="AS42" s="5" t="n"/>
-      <c r="BI42" s="5" t="n"/>
+      <c r="T42" s="5" t="n"/>
+      <c r="AT42" s="6" t="n"/>
+      <c r="BJ42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
-      <c r="R43" s="5" t="n"/>
+      <c r="B43" s="6" t="n"/>
       <c r="S43" s="6" t="n"/>
-      <c r="AS43" s="5" t="n"/>
-      <c r="BI43" s="5" t="n"/>
+      <c r="T43" s="5" t="n"/>
+      <c r="AT43" s="6" t="n"/>
+      <c r="BJ43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n"/>
-      <c r="R44" s="5" t="n"/>
+      <c r="B44" s="6" t="n"/>
       <c r="S44" s="6" t="n"/>
-      <c r="AS44" s="5" t="n"/>
-      <c r="BI44" s="5" t="n"/>
+      <c r="T44" s="5" t="n"/>
+      <c r="AT44" s="6" t="n"/>
+      <c r="BJ44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n"/>
-      <c r="R45" s="5" t="n"/>
+      <c r="B45" s="6" t="n"/>
       <c r="S45" s="6" t="n"/>
-      <c r="AS45" s="5" t="n"/>
-      <c r="BI45" s="5" t="n"/>
+      <c r="T45" s="5" t="n"/>
+      <c r="AT45" s="6" t="n"/>
+      <c r="BJ45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n"/>
-      <c r="R46" s="5" t="n"/>
+      <c r="B46" s="6" t="n"/>
       <c r="S46" s="6" t="n"/>
-      <c r="AS46" s="5" t="n"/>
-      <c r="BI46" s="5" t="n"/>
+      <c r="T46" s="5" t="n"/>
+      <c r="AT46" s="6" t="n"/>
+      <c r="BJ46" s="6" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n"/>
-      <c r="R47" s="5" t="n"/>
+      <c r="B47" s="6" t="n"/>
       <c r="S47" s="6" t="n"/>
-      <c r="AS47" s="5" t="n"/>
-      <c r="BI47" s="5" t="n"/>
+      <c r="T47" s="5" t="n"/>
+      <c r="AT47" s="6" t="n"/>
+      <c r="BJ47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n"/>
-      <c r="R48" s="5" t="n"/>
+      <c r="B48" s="6" t="n"/>
       <c r="S48" s="6" t="n"/>
-      <c r="AS48" s="5" t="n"/>
-      <c r="BI48" s="5" t="n"/>
+      <c r="T48" s="5" t="n"/>
+      <c r="AT48" s="6" t="n"/>
+      <c r="BJ48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n"/>
-      <c r="R49" s="5" t="n"/>
+      <c r="B49" s="6" t="n"/>
       <c r="S49" s="6" t="n"/>
-      <c r="AS49" s="5" t="n"/>
-      <c r="BI49" s="5" t="n"/>
+      <c r="T49" s="5" t="n"/>
+      <c r="AT49" s="6" t="n"/>
+      <c r="BJ49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n"/>
-      <c r="R50" s="5" t="n"/>
+      <c r="B50" s="6" t="n"/>
       <c r="S50" s="6" t="n"/>
-      <c r="AS50" s="5" t="n"/>
-      <c r="BI50" s="5" t="n"/>
+      <c r="T50" s="5" t="n"/>
+      <c r="AT50" s="6" t="n"/>
+      <c r="BJ50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>
-      <c r="R51" s="5" t="n"/>
+      <c r="B51" s="6" t="n"/>
       <c r="S51" s="6" t="n"/>
-      <c r="AS51" s="5" t="n"/>
-      <c r="BI51" s="5" t="n"/>
+      <c r="T51" s="5" t="n"/>
+      <c r="AT51" s="6" t="n"/>
+      <c r="BJ51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n"/>
-      <c r="R52" s="5" t="n"/>
+      <c r="B52" s="6" t="n"/>
       <c r="S52" s="6" t="n"/>
-      <c r="AS52" s="5" t="n"/>
-      <c r="BI52" s="5" t="n"/>
+      <c r="T52" s="5" t="n"/>
+      <c r="AT52" s="6" t="n"/>
+      <c r="BJ52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
-      <c r="R53" s="5" t="n"/>
+      <c r="B53" s="6" t="n"/>
       <c r="S53" s="6" t="n"/>
-      <c r="AS53" s="5" t="n"/>
-      <c r="BI53" s="5" t="n"/>
+      <c r="T53" s="5" t="n"/>
+      <c r="AT53" s="6" t="n"/>
+      <c r="BJ53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n"/>
-      <c r="R54" s="5" t="n"/>
+      <c r="B54" s="6" t="n"/>
       <c r="S54" s="6" t="n"/>
-      <c r="AS54" s="5" t="n"/>
-      <c r="BI54" s="5" t="n"/>
+      <c r="T54" s="5" t="n"/>
+      <c r="AT54" s="6" t="n"/>
+      <c r="BJ54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n"/>
-      <c r="R55" s="5" t="n"/>
+      <c r="B55" s="6" t="n"/>
       <c r="S55" s="6" t="n"/>
-      <c r="AS55" s="5" t="n"/>
-      <c r="BI55" s="5" t="n"/>
+      <c r="T55" s="5" t="n"/>
+      <c r="AT55" s="6" t="n"/>
+      <c r="BJ55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n"/>
-      <c r="R56" s="5" t="n"/>
+      <c r="B56" s="6" t="n"/>
       <c r="S56" s="6" t="n"/>
-      <c r="AS56" s="5" t="n"/>
-      <c r="BI56" s="5" t="n"/>
+      <c r="T56" s="5" t="n"/>
+      <c r="AT56" s="6" t="n"/>
+      <c r="BJ56" s="6" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n"/>
-      <c r="R57" s="5" t="n"/>
+      <c r="B57" s="6" t="n"/>
       <c r="S57" s="6" t="n"/>
-      <c r="AS57" s="5" t="n"/>
-      <c r="BI57" s="5" t="n"/>
+      <c r="T57" s="5" t="n"/>
+      <c r="AT57" s="6" t="n"/>
+      <c r="BJ57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n"/>
-      <c r="R58" s="5" t="n"/>
+      <c r="B58" s="6" t="n"/>
       <c r="S58" s="6" t="n"/>
-      <c r="AS58" s="5" t="n"/>
-      <c r="BI58" s="5" t="n"/>
+      <c r="T58" s="5" t="n"/>
+      <c r="AT58" s="6" t="n"/>
+      <c r="BJ58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n"/>
-      <c r="R59" s="5" t="n"/>
+      <c r="B59" s="6" t="n"/>
       <c r="S59" s="6" t="n"/>
-      <c r="AS59" s="5" t="n"/>
-      <c r="BI59" s="5" t="n"/>
+      <c r="T59" s="5" t="n"/>
+      <c r="AT59" s="6" t="n"/>
+      <c r="BJ59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n"/>
-      <c r="R60" s="5" t="n"/>
+      <c r="B60" s="6" t="n"/>
       <c r="S60" s="6" t="n"/>
-      <c r="AS60" s="5" t="n"/>
-      <c r="BI60" s="5" t="n"/>
+      <c r="T60" s="5" t="n"/>
+      <c r="AT60" s="6" t="n"/>
+      <c r="BJ60" s="6" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n"/>
-      <c r="R61" s="5" t="n"/>
+      <c r="B61" s="6" t="n"/>
       <c r="S61" s="6" t="n"/>
-      <c r="AS61" s="5" t="n"/>
-      <c r="BI61" s="5" t="n"/>
+      <c r="T61" s="5" t="n"/>
+      <c r="AT61" s="6" t="n"/>
+      <c r="BJ61" s="6" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n"/>
-      <c r="R62" s="5" t="n"/>
+      <c r="B62" s="6" t="n"/>
       <c r="S62" s="6" t="n"/>
-      <c r="AS62" s="5" t="n"/>
-      <c r="BI62" s="5" t="n"/>
+      <c r="T62" s="5" t="n"/>
+      <c r="AT62" s="6" t="n"/>
+      <c r="BJ62" s="6" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n"/>
-      <c r="R63" s="5" t="n"/>
+      <c r="B63" s="6" t="n"/>
       <c r="S63" s="6" t="n"/>
-      <c r="AS63" s="5" t="n"/>
-      <c r="BI63" s="5" t="n"/>
+      <c r="T63" s="5" t="n"/>
+      <c r="AT63" s="6" t="n"/>
+      <c r="BJ63" s="6" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n"/>
-      <c r="R64" s="5" t="n"/>
+      <c r="B64" s="6" t="n"/>
       <c r="S64" s="6" t="n"/>
-      <c r="AS64" s="5" t="n"/>
-      <c r="BI64" s="5" t="n"/>
+      <c r="T64" s="5" t="n"/>
+      <c r="AT64" s="6" t="n"/>
+      <c r="BJ64" s="6" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n"/>
-      <c r="R65" s="5" t="n"/>
+      <c r="B65" s="6" t="n"/>
       <c r="S65" s="6" t="n"/>
-      <c r="AS65" s="5" t="n"/>
-      <c r="BI65" s="5" t="n"/>
+      <c r="T65" s="5" t="n"/>
+      <c r="AT65" s="6" t="n"/>
+      <c r="BJ65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n"/>
-      <c r="R66" s="5" t="n"/>
+      <c r="B66" s="6" t="n"/>
       <c r="S66" s="6" t="n"/>
-      <c r="AS66" s="5" t="n"/>
-      <c r="BI66" s="5" t="n"/>
+      <c r="T66" s="5" t="n"/>
+      <c r="AT66" s="6" t="n"/>
+      <c r="BJ66" s="6" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n"/>
-      <c r="R67" s="5" t="n"/>
+      <c r="B67" s="6" t="n"/>
       <c r="S67" s="6" t="n"/>
-      <c r="AS67" s="5" t="n"/>
-      <c r="BI67" s="5" t="n"/>
+      <c r="T67" s="5" t="n"/>
+      <c r="AT67" s="6" t="n"/>
+      <c r="BJ67" s="6" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n"/>
-      <c r="R68" s="5" t="n"/>
+      <c r="B68" s="6" t="n"/>
       <c r="S68" s="6" t="n"/>
-      <c r="AS68" s="5" t="n"/>
-      <c r="BI68" s="5" t="n"/>
+      <c r="T68" s="5" t="n"/>
+      <c r="AT68" s="6" t="n"/>
+      <c r="BJ68" s="6" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n"/>
-      <c r="R69" s="5" t="n"/>
+      <c r="B69" s="6" t="n"/>
       <c r="S69" s="6" t="n"/>
-      <c r="AS69" s="5" t="n"/>
-      <c r="BI69" s="5" t="n"/>
+      <c r="T69" s="5" t="n"/>
+      <c r="AT69" s="6" t="n"/>
+      <c r="BJ69" s="6" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n"/>
-      <c r="R70" s="5" t="n"/>
+      <c r="B70" s="6" t="n"/>
       <c r="S70" s="6" t="n"/>
-      <c r="AS70" s="5" t="n"/>
-      <c r="BI70" s="5" t="n"/>
+      <c r="T70" s="5" t="n"/>
+      <c r="AT70" s="6" t="n"/>
+      <c r="BJ70" s="6" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n"/>
-      <c r="R71" s="5" t="n"/>
+      <c r="B71" s="6" t="n"/>
       <c r="S71" s="6" t="n"/>
-      <c r="AS71" s="5" t="n"/>
-      <c r="BI71" s="5" t="n"/>
+      <c r="T71" s="5" t="n"/>
+      <c r="AT71" s="6" t="n"/>
+      <c r="BJ71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n"/>
-      <c r="R72" s="5" t="n"/>
+      <c r="B72" s="6" t="n"/>
       <c r="S72" s="6" t="n"/>
-      <c r="AS72" s="5" t="n"/>
-      <c r="BI72" s="5" t="n"/>
+      <c r="T72" s="5" t="n"/>
+      <c r="AT72" s="6" t="n"/>
+      <c r="BJ72" s="6" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n"/>
-      <c r="R73" s="5" t="n"/>
+      <c r="B73" s="6" t="n"/>
       <c r="S73" s="6" t="n"/>
-      <c r="AS73" s="5" t="n"/>
-      <c r="BI73" s="5" t="n"/>
+      <c r="T73" s="5" t="n"/>
+      <c r="AT73" s="6" t="n"/>
+      <c r="BJ73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n"/>
-      <c r="R74" s="5" t="n"/>
+      <c r="B74" s="6" t="n"/>
       <c r="S74" s="6" t="n"/>
-      <c r="AS74" s="5" t="n"/>
-      <c r="BI74" s="5" t="n"/>
+      <c r="T74" s="5" t="n"/>
+      <c r="AT74" s="6" t="n"/>
+      <c r="BJ74" s="6" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n"/>
-      <c r="R75" s="5" t="n"/>
+      <c r="B75" s="6" t="n"/>
       <c r="S75" s="6" t="n"/>
-      <c r="AS75" s="5" t="n"/>
-      <c r="BI75" s="5" t="n"/>
+      <c r="T75" s="5" t="n"/>
+      <c r="AT75" s="6" t="n"/>
+      <c r="BJ75" s="6" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n"/>
-      <c r="R76" s="5" t="n"/>
+      <c r="B76" s="6" t="n"/>
       <c r="S76" s="6" t="n"/>
-      <c r="AS76" s="5" t="n"/>
-      <c r="BI76" s="5" t="n"/>
+      <c r="T76" s="5" t="n"/>
+      <c r="AT76" s="6" t="n"/>
+      <c r="BJ76" s="6" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n"/>
-      <c r="R77" s="5" t="n"/>
+      <c r="B77" s="6" t="n"/>
       <c r="S77" s="6" t="n"/>
-      <c r="AS77" s="5" t="n"/>
-      <c r="BI77" s="5" t="n"/>
+      <c r="T77" s="5" t="n"/>
+      <c r="AT77" s="6" t="n"/>
+      <c r="BJ77" s="6" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n"/>
-      <c r="R78" s="5" t="n"/>
+      <c r="B78" s="6" t="n"/>
       <c r="S78" s="6" t="n"/>
-      <c r="AS78" s="5" t="n"/>
-      <c r="BI78" s="5" t="n"/>
+      <c r="T78" s="5" t="n"/>
+      <c r="AT78" s="6" t="n"/>
+      <c r="BJ78" s="6" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n"/>
-      <c r="R79" s="5" t="n"/>
+      <c r="B79" s="6" t="n"/>
       <c r="S79" s="6" t="n"/>
-      <c r="AS79" s="5" t="n"/>
-      <c r="BI79" s="5" t="n"/>
+      <c r="T79" s="5" t="n"/>
+      <c r="AT79" s="6" t="n"/>
+      <c r="BJ79" s="6" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n"/>
-      <c r="R80" s="5" t="n"/>
+      <c r="B80" s="6" t="n"/>
       <c r="S80" s="6" t="n"/>
-      <c r="AS80" s="5" t="n"/>
-      <c r="BI80" s="5" t="n"/>
+      <c r="T80" s="5" t="n"/>
+      <c r="AT80" s="6" t="n"/>
+      <c r="BJ80" s="6" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n"/>
-      <c r="R81" s="5" t="n"/>
+      <c r="B81" s="6" t="n"/>
       <c r="S81" s="6" t="n"/>
-      <c r="AS81" s="5" t="n"/>
-      <c r="BI81" s="5" t="n"/>
+      <c r="T81" s="5" t="n"/>
+      <c r="AT81" s="6" t="n"/>
+      <c r="BJ81" s="6" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n"/>
-      <c r="R82" s="5" t="n"/>
+      <c r="B82" s="6" t="n"/>
       <c r="S82" s="6" t="n"/>
-      <c r="AS82" s="5" t="n"/>
-      <c r="BI82" s="5" t="n"/>
+      <c r="T82" s="5" t="n"/>
+      <c r="AT82" s="6" t="n"/>
+      <c r="BJ82" s="6" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n"/>
-      <c r="R83" s="5" t="n"/>
+      <c r="B83" s="6" t="n"/>
       <c r="S83" s="6" t="n"/>
-      <c r="AS83" s="5" t="n"/>
-      <c r="BI83" s="5" t="n"/>
+      <c r="T83" s="5" t="n"/>
+      <c r="AT83" s="6" t="n"/>
+      <c r="BJ83" s="6" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n"/>
-      <c r="R84" s="5" t="n"/>
+      <c r="B84" s="6" t="n"/>
       <c r="S84" s="6" t="n"/>
-      <c r="AS84" s="5" t="n"/>
-      <c r="BI84" s="5" t="n"/>
+      <c r="T84" s="5" t="n"/>
+      <c r="AT84" s="6" t="n"/>
+      <c r="BJ84" s="6" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n"/>
-      <c r="R85" s="5" t="n"/>
+      <c r="B85" s="6" t="n"/>
       <c r="S85" s="6" t="n"/>
-      <c r="AS85" s="5" t="n"/>
-      <c r="BI85" s="5" t="n"/>
+      <c r="T85" s="5" t="n"/>
+      <c r="AT85" s="6" t="n"/>
+      <c r="BJ85" s="6" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="n"/>
-      <c r="R86" s="5" t="n"/>
+      <c r="B86" s="6" t="n"/>
       <c r="S86" s="6" t="n"/>
-      <c r="AS86" s="5" t="n"/>
-      <c r="BI86" s="5" t="n"/>
+      <c r="T86" s="5" t="n"/>
+      <c r="AT86" s="6" t="n"/>
+      <c r="BJ86" s="6" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n"/>
-      <c r="R87" s="5" t="n"/>
+      <c r="B87" s="6" t="n"/>
       <c r="S87" s="6" t="n"/>
-      <c r="AS87" s="5" t="n"/>
-      <c r="BI87" s="5" t="n"/>
+      <c r="T87" s="5" t="n"/>
+      <c r="AT87" s="6" t="n"/>
+      <c r="BJ87" s="6" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="5" t="n"/>
-      <c r="R88" s="5" t="n"/>
+      <c r="B88" s="6" t="n"/>
       <c r="S88" s="6" t="n"/>
-      <c r="AS88" s="5" t="n"/>
-      <c r="BI88" s="5" t="n"/>
+      <c r="T88" s="5" t="n"/>
+      <c r="AT88" s="6" t="n"/>
+      <c r="BJ88" s="6" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="5" t="n"/>
-      <c r="R89" s="5" t="n"/>
+      <c r="B89" s="6" t="n"/>
       <c r="S89" s="6" t="n"/>
-      <c r="AS89" s="5" t="n"/>
-      <c r="BI89" s="5" t="n"/>
+      <c r="T89" s="5" t="n"/>
+      <c r="AT89" s="6" t="n"/>
+      <c r="BJ89" s="6" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="n"/>
-      <c r="R90" s="5" t="n"/>
+      <c r="B90" s="6" t="n"/>
       <c r="S90" s="6" t="n"/>
-      <c r="AS90" s="5" t="n"/>
-      <c r="BI90" s="5" t="n"/>
+      <c r="T90" s="5" t="n"/>
+      <c r="AT90" s="6" t="n"/>
+      <c r="BJ90" s="6" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="5" t="n"/>
-      <c r="R91" s="5" t="n"/>
+      <c r="B91" s="6" t="n"/>
       <c r="S91" s="6" t="n"/>
-      <c r="AS91" s="5" t="n"/>
-      <c r="BI91" s="5" t="n"/>
+      <c r="T91" s="5" t="n"/>
+      <c r="AT91" s="6" t="n"/>
+      <c r="BJ91" s="6" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="n"/>
-      <c r="R92" s="5" t="n"/>
+      <c r="B92" s="6" t="n"/>
       <c r="S92" s="6" t="n"/>
-      <c r="AS92" s="5" t="n"/>
-      <c r="BI92" s="5" t="n"/>
+      <c r="T92" s="5" t="n"/>
+      <c r="AT92" s="6" t="n"/>
+      <c r="BJ92" s="6" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="5" t="n"/>
-      <c r="R93" s="5" t="n"/>
+      <c r="B93" s="6" t="n"/>
       <c r="S93" s="6" t="n"/>
-      <c r="AS93" s="5" t="n"/>
-      <c r="BI93" s="5" t="n"/>
+      <c r="T93" s="5" t="n"/>
+      <c r="AT93" s="6" t="n"/>
+      <c r="BJ93" s="6" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n"/>
-      <c r="R94" s="5" t="n"/>
+      <c r="B94" s="6" t="n"/>
       <c r="S94" s="6" t="n"/>
-      <c r="AS94" s="5" t="n"/>
-      <c r="BI94" s="5" t="n"/>
+      <c r="T94" s="5" t="n"/>
+      <c r="AT94" s="6" t="n"/>
+      <c r="BJ94" s="6" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="5" t="n"/>
-      <c r="R95" s="5" t="n"/>
+      <c r="B95" s="6" t="n"/>
       <c r="S95" s="6" t="n"/>
-      <c r="AS95" s="5" t="n"/>
-      <c r="BI95" s="5" t="n"/>
+      <c r="T95" s="5" t="n"/>
+      <c r="AT95" s="6" t="n"/>
+      <c r="BJ95" s="6" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="n"/>
-      <c r="R96" s="5" t="n"/>
+      <c r="B96" s="6" t="n"/>
       <c r="S96" s="6" t="n"/>
-      <c r="AS96" s="5" t="n"/>
-      <c r="BI96" s="5" t="n"/>
+      <c r="T96" s="5" t="n"/>
+      <c r="AT96" s="6" t="n"/>
+      <c r="BJ96" s="6" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="5" t="n"/>
-      <c r="R97" s="5" t="n"/>
+      <c r="B97" s="6" t="n"/>
       <c r="S97" s="6" t="n"/>
-      <c r="AS97" s="5" t="n"/>
-      <c r="BI97" s="5" t="n"/>
+      <c r="T97" s="5" t="n"/>
+      <c r="AT97" s="6" t="n"/>
+      <c r="BJ97" s="6" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n"/>
-      <c r="R98" s="5" t="n"/>
+      <c r="B98" s="6" t="n"/>
       <c r="S98" s="6" t="n"/>
-      <c r="AS98" s="5" t="n"/>
-      <c r="BI98" s="5" t="n"/>
+      <c r="T98" s="5" t="n"/>
+      <c r="AT98" s="6" t="n"/>
+      <c r="BJ98" s="6" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="5" t="n"/>
-      <c r="R99" s="5" t="n"/>
+      <c r="B99" s="6" t="n"/>
       <c r="S99" s="6" t="n"/>
-      <c r="AS99" s="5" t="n"/>
-      <c r="BI99" s="5" t="n"/>
+      <c r="T99" s="5" t="n"/>
+      <c r="AT99" s="6" t="n"/>
+      <c r="BJ99" s="6" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="5" t="n"/>
-      <c r="R100" s="5" t="n"/>
+      <c r="B100" s="6" t="n"/>
       <c r="S100" s="6" t="n"/>
-      <c r="AS100" s="5" t="n"/>
-      <c r="BI100" s="5" t="n"/>
+      <c r="T100" s="5" t="n"/>
+      <c r="AT100" s="6" t="n"/>
+      <c r="BJ100" s="6" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="n"/>
-      <c r="R101" s="5" t="n"/>
+      <c r="B101" s="6" t="n"/>
       <c r="S101" s="6" t="n"/>
-      <c r="AS101" s="5" t="n"/>
-      <c r="BI101" s="5" t="n"/>
+      <c r="T101" s="5" t="n"/>
+      <c r="AT101" s="6" t="n"/>
+      <c r="BJ101" s="6" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="5" t="n"/>
-      <c r="R102" s="5" t="n"/>
+      <c r="B102" s="6" t="n"/>
       <c r="S102" s="6" t="n"/>
-      <c r="AS102" s="5" t="n"/>
-      <c r="BI102" s="5" t="n"/>
+      <c r="T102" s="5" t="n"/>
+      <c r="AT102" s="6" t="n"/>
+      <c r="BJ102" s="6" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="5" t="n"/>
-      <c r="R103" s="5" t="n"/>
+      <c r="B103" s="6" t="n"/>
       <c r="S103" s="6" t="n"/>
-      <c r="AS103" s="5" t="n"/>
-      <c r="BI103" s="5" t="n"/>
+      <c r="T103" s="5" t="n"/>
+      <c r="AT103" s="6" t="n"/>
+      <c r="BJ103" s="6" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="n"/>
-      <c r="R104" s="5" t="n"/>
+      <c r="B104" s="6" t="n"/>
       <c r="S104" s="6" t="n"/>
-      <c r="AS104" s="5" t="n"/>
-      <c r="BI104" s="5" t="n"/>
+      <c r="T104" s="5" t="n"/>
+      <c r="AT104" s="6" t="n"/>
+      <c r="BJ104" s="6" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="5" t="n"/>
-      <c r="R105" s="5" t="n"/>
+      <c r="B105" s="6" t="n"/>
       <c r="S105" s="6" t="n"/>
-      <c r="AS105" s="5" t="n"/>
-      <c r="BI105" s="5" t="n"/>
+      <c r="T105" s="5" t="n"/>
+      <c r="AT105" s="6" t="n"/>
+      <c r="BJ105" s="6" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="n"/>
-      <c r="R106" s="5" t="n"/>
+      <c r="B106" s="6" t="n"/>
       <c r="S106" s="6" t="n"/>
-      <c r="AS106" s="5" t="n"/>
-      <c r="BI106" s="5" t="n"/>
+      <c r="T106" s="5" t="n"/>
+      <c r="AT106" s="6" t="n"/>
+      <c r="BJ106" s="6" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n"/>
-      <c r="R107" s="5" t="n"/>
+      <c r="B107" s="6" t="n"/>
       <c r="S107" s="6" t="n"/>
-      <c r="AS107" s="5" t="n"/>
-      <c r="BI107" s="5" t="n"/>
+      <c r="T107" s="5" t="n"/>
+      <c r="AT107" s="6" t="n"/>
+      <c r="BJ107" s="6" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="n"/>
-      <c r="R108" s="5" t="n"/>
+      <c r="B108" s="6" t="n"/>
       <c r="S108" s="6" t="n"/>
-      <c r="AS108" s="5" t="n"/>
-      <c r="BI108" s="5" t="n"/>
+      <c r="T108" s="5" t="n"/>
+      <c r="AT108" s="6" t="n"/>
+      <c r="BJ108" s="6" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="5" t="n"/>
-      <c r="R109" s="5" t="n"/>
+      <c r="B109" s="6" t="n"/>
       <c r="S109" s="6" t="n"/>
-      <c r="AS109" s="5" t="n"/>
-      <c r="BI109" s="5" t="n"/>
+      <c r="T109" s="5" t="n"/>
+      <c r="AT109" s="6" t="n"/>
+      <c r="BJ109" s="6" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="n"/>
-      <c r="R110" s="5" t="n"/>
+      <c r="B110" s="6" t="n"/>
       <c r="S110" s="6" t="n"/>
-      <c r="AS110" s="5" t="n"/>
-      <c r="BI110" s="5" t="n"/>
+      <c r="T110" s="5" t="n"/>
+      <c r="AT110" s="6" t="n"/>
+      <c r="BJ110" s="6" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="5" t="n"/>
-      <c r="R111" s="5" t="n"/>
+      <c r="B111" s="6" t="n"/>
       <c r="S111" s="6" t="n"/>
-      <c r="AS111" s="5" t="n"/>
-      <c r="BI111" s="5" t="n"/>
+      <c r="T111" s="5" t="n"/>
+      <c r="AT111" s="6" t="n"/>
+      <c r="BJ111" s="6" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="n"/>
-      <c r="R112" s="5" t="n"/>
+      <c r="B112" s="6" t="n"/>
       <c r="S112" s="6" t="n"/>
-      <c r="AS112" s="5" t="n"/>
-      <c r="BI112" s="5" t="n"/>
+      <c r="T112" s="5" t="n"/>
+      <c r="AT112" s="6" t="n"/>
+      <c r="BJ112" s="6" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="5" t="n"/>
-      <c r="R113" s="5" t="n"/>
+      <c r="B113" s="6" t="n"/>
       <c r="S113" s="6" t="n"/>
-      <c r="AS113" s="5" t="n"/>
-      <c r="BI113" s="5" t="n"/>
+      <c r="T113" s="5" t="n"/>
+      <c r="AT113" s="6" t="n"/>
+      <c r="BJ113" s="6" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="5" t="n"/>
-      <c r="R114" s="5" t="n"/>
+      <c r="B114" s="6" t="n"/>
       <c r="S114" s="6" t="n"/>
-      <c r="AS114" s="5" t="n"/>
-      <c r="BI114" s="5" t="n"/>
+      <c r="T114" s="5" t="n"/>
+      <c r="AT114" s="6" t="n"/>
+      <c r="BJ114" s="6" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="5" t="n"/>
-      <c r="R115" s="5" t="n"/>
+      <c r="B115" s="6" t="n"/>
       <c r="S115" s="6" t="n"/>
-      <c r="AS115" s="5" t="n"/>
-      <c r="BI115" s="5" t="n"/>
+      <c r="T115" s="5" t="n"/>
+      <c r="AT115" s="6" t="n"/>
+      <c r="BJ115" s="6" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="5" t="n"/>
-      <c r="R116" s="5" t="n"/>
+      <c r="B116" s="6" t="n"/>
       <c r="S116" s="6" t="n"/>
-      <c r="AS116" s="5" t="n"/>
-      <c r="BI116" s="5" t="n"/>
+      <c r="T116" s="5" t="n"/>
+      <c r="AT116" s="6" t="n"/>
+      <c r="BJ116" s="6" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="5" t="n"/>
-      <c r="R117" s="5" t="n"/>
+      <c r="B117" s="6" t="n"/>
       <c r="S117" s="6" t="n"/>
-      <c r="AS117" s="5" t="n"/>
-      <c r="BI117" s="5" t="n"/>
+      <c r="T117" s="5" t="n"/>
+      <c r="AT117" s="6" t="n"/>
+      <c r="BJ117" s="6" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="5" t="n"/>
-      <c r="R118" s="5" t="n"/>
+      <c r="B118" s="6" t="n"/>
       <c r="S118" s="6" t="n"/>
-      <c r="AS118" s="5" t="n"/>
-      <c r="BI118" s="5" t="n"/>
+      <c r="T118" s="5" t="n"/>
+      <c r="AT118" s="6" t="n"/>
+      <c r="BJ118" s="6" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="5" t="n"/>
-      <c r="R119" s="5" t="n"/>
+      <c r="B119" s="6" t="n"/>
       <c r="S119" s="6" t="n"/>
-      <c r="AS119" s="5" t="n"/>
-      <c r="BI119" s="5" t="n"/>
+      <c r="T119" s="5" t="n"/>
+      <c r="AT119" s="6" t="n"/>
+      <c r="BJ119" s="6" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="n"/>
-      <c r="R120" s="5" t="n"/>
+      <c r="B120" s="6" t="n"/>
       <c r="S120" s="6" t="n"/>
-      <c r="AS120" s="5" t="n"/>
-      <c r="BI120" s="5" t="n"/>
+      <c r="T120" s="5" t="n"/>
+      <c r="AT120" s="6" t="n"/>
+      <c r="BJ120" s="6" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="5" t="n"/>
-      <c r="R121" s="5" t="n"/>
+      <c r="B121" s="6" t="n"/>
       <c r="S121" s="6" t="n"/>
-      <c r="AS121" s="5" t="n"/>
-      <c r="BI121" s="5" t="n"/>
+      <c r="T121" s="5" t="n"/>
+      <c r="AT121" s="6" t="n"/>
+      <c r="BJ121" s="6" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="5" t="n"/>
-      <c r="R122" s="5" t="n"/>
+      <c r="B122" s="6" t="n"/>
       <c r="S122" s="6" t="n"/>
-      <c r="AS122" s="5" t="n"/>
-      <c r="BI122" s="5" t="n"/>
+      <c r="T122" s="5" t="n"/>
+      <c r="AT122" s="6" t="n"/>
+      <c r="BJ122" s="6" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="5" t="n"/>
-      <c r="R123" s="5" t="n"/>
+      <c r="B123" s="6" t="n"/>
       <c r="S123" s="6" t="n"/>
-      <c r="AS123" s="5" t="n"/>
-      <c r="BI123" s="5" t="n"/>
+      <c r="T123" s="5" t="n"/>
+      <c r="AT123" s="6" t="n"/>
+      <c r="BJ123" s="6" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="5" t="n"/>
-      <c r="R124" s="5" t="n"/>
+      <c r="B124" s="6" t="n"/>
       <c r="S124" s="6" t="n"/>
-      <c r="AS124" s="5" t="n"/>
-      <c r="BI124" s="5" t="n"/>
+      <c r="T124" s="5" t="n"/>
+      <c r="AT124" s="6" t="n"/>
+      <c r="BJ124" s="6" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="5" t="n"/>
-      <c r="R125" s="5" t="n"/>
+      <c r="B125" s="6" t="n"/>
       <c r="S125" s="6" t="n"/>
-      <c r="AS125" s="5" t="n"/>
-      <c r="BI125" s="5" t="n"/>
+      <c r="T125" s="5" t="n"/>
+      <c r="AT125" s="6" t="n"/>
+      <c r="BJ125" s="6" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="n"/>
-      <c r="R126" s="5" t="n"/>
+      <c r="B126" s="6" t="n"/>
       <c r="S126" s="6" t="n"/>
-      <c r="AS126" s="5" t="n"/>
-      <c r="BI126" s="5" t="n"/>
+      <c r="T126" s="5" t="n"/>
+      <c r="AT126" s="6" t="n"/>
+      <c r="BJ126" s="6" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="5" t="n"/>
-      <c r="R127" s="5" t="n"/>
+      <c r="B127" s="6" t="n"/>
       <c r="S127" s="6" t="n"/>
-      <c r="AS127" s="5" t="n"/>
-      <c r="BI127" s="5" t="n"/>
+      <c r="T127" s="5" t="n"/>
+      <c r="AT127" s="6" t="n"/>
+      <c r="BJ127" s="6" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="5" t="n"/>
-      <c r="R128" s="5" t="n"/>
+      <c r="B128" s="6" t="n"/>
       <c r="S128" s="6" t="n"/>
-      <c r="AS128" s="5" t="n"/>
-      <c r="BI128" s="5" t="n"/>
+      <c r="T128" s="5" t="n"/>
+      <c r="AT128" s="6" t="n"/>
+      <c r="BJ128" s="6" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="5" t="n"/>
-      <c r="R129" s="5" t="n"/>
+      <c r="B129" s="6" t="n"/>
       <c r="S129" s="6" t="n"/>
-      <c r="AS129" s="5" t="n"/>
-      <c r="BI129" s="5" t="n"/>
+      <c r="T129" s="5" t="n"/>
+      <c r="AT129" s="6" t="n"/>
+      <c r="BJ129" s="6" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="n"/>
-      <c r="R130" s="5" t="n"/>
+      <c r="B130" s="6" t="n"/>
       <c r="S130" s="6" t="n"/>
-      <c r="AS130" s="5" t="n"/>
-      <c r="BI130" s="5" t="n"/>
+      <c r="T130" s="5" t="n"/>
+      <c r="AT130" s="6" t="n"/>
+      <c r="BJ130" s="6" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="5" t="n"/>
-      <c r="R131" s="5" t="n"/>
+      <c r="B131" s="6" t="n"/>
       <c r="S131" s="6" t="n"/>
-      <c r="AS131" s="5" t="n"/>
-      <c r="BI131" s="5" t="n"/>
+      <c r="T131" s="5" t="n"/>
+      <c r="AT131" s="6" t="n"/>
+      <c r="BJ131" s="6" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="5" t="n"/>
-      <c r="R132" s="5" t="n"/>
+      <c r="B132" s="6" t="n"/>
       <c r="S132" s="6" t="n"/>
-      <c r="AS132" s="5" t="n"/>
-      <c r="BI132" s="5" t="n"/>
+      <c r="T132" s="5" t="n"/>
+      <c r="AT132" s="6" t="n"/>
+      <c r="BJ132" s="6" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="5" t="n"/>
-      <c r="R133" s="5" t="n"/>
+      <c r="B133" s="6" t="n"/>
       <c r="S133" s="6" t="n"/>
-      <c r="AS133" s="5" t="n"/>
-      <c r="BI133" s="5" t="n"/>
+      <c r="T133" s="5" t="n"/>
+      <c r="AT133" s="6" t="n"/>
+      <c r="BJ133" s="6" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="5" t="n"/>
-      <c r="R134" s="5" t="n"/>
+      <c r="B134" s="6" t="n"/>
       <c r="S134" s="6" t="n"/>
-      <c r="AS134" s="5" t="n"/>
-      <c r="BI134" s="5" t="n"/>
+      <c r="T134" s="5" t="n"/>
+      <c r="AT134" s="6" t="n"/>
+      <c r="BJ134" s="6" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="5" t="n"/>
-      <c r="R135" s="5" t="n"/>
+      <c r="B135" s="6" t="n"/>
       <c r="S135" s="6" t="n"/>
-      <c r="AS135" s="5" t="n"/>
-      <c r="BI135" s="5" t="n"/>
+      <c r="T135" s="5" t="n"/>
+      <c r="AT135" s="6" t="n"/>
+      <c r="BJ135" s="6" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="5" t="n"/>
-      <c r="R136" s="5" t="n"/>
+      <c r="B136" s="6" t="n"/>
       <c r="S136" s="6" t="n"/>
-      <c r="AS136" s="5" t="n"/>
-      <c r="BI136" s="5" t="n"/>
+      <c r="T136" s="5" t="n"/>
+      <c r="AT136" s="6" t="n"/>
+      <c r="BJ136" s="6" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="5" t="n"/>
-      <c r="R137" s="5" t="n"/>
+      <c r="B137" s="6" t="n"/>
       <c r="S137" s="6" t="n"/>
-      <c r="AS137" s="5" t="n"/>
-      <c r="BI137" s="5" t="n"/>
+      <c r="T137" s="5" t="n"/>
+      <c r="AT137" s="6" t="n"/>
+      <c r="BJ137" s="6" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="n"/>
-      <c r="R138" s="5" t="n"/>
+      <c r="B138" s="6" t="n"/>
       <c r="S138" s="6" t="n"/>
-      <c r="AS138" s="5" t="n"/>
-      <c r="BI138" s="5" t="n"/>
+      <c r="T138" s="5" t="n"/>
+      <c r="AT138" s="6" t="n"/>
+      <c r="BJ138" s="6" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="5" t="n"/>
-      <c r="R139" s="5" t="n"/>
+      <c r="B139" s="6" t="n"/>
       <c r="S139" s="6" t="n"/>
-      <c r="AS139" s="5" t="n"/>
-      <c r="BI139" s="5" t="n"/>
+      <c r="T139" s="5" t="n"/>
+      <c r="AT139" s="6" t="n"/>
+      <c r="BJ139" s="6" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="5" t="n"/>
-      <c r="R140" s="5" t="n"/>
+      <c r="B140" s="6" t="n"/>
       <c r="S140" s="6" t="n"/>
-      <c r="AS140" s="5" t="n"/>
-      <c r="BI140" s="5" t="n"/>
+      <c r="T140" s="5" t="n"/>
+      <c r="AT140" s="6" t="n"/>
+      <c r="BJ140" s="6" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="5" t="n"/>
-      <c r="R141" s="5" t="n"/>
+      <c r="B141" s="6" t="n"/>
       <c r="S141" s="6" t="n"/>
-      <c r="AS141" s="5" t="n"/>
-      <c r="BI141" s="5" t="n"/>
+      <c r="T141" s="5" t="n"/>
+      <c r="AT141" s="6" t="n"/>
+      <c r="BJ141" s="6" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="5" t="n"/>
-      <c r="R142" s="5" t="n"/>
+      <c r="B142" s="6" t="n"/>
       <c r="S142" s="6" t="n"/>
-      <c r="AS142" s="5" t="n"/>
-      <c r="BI142" s="5" t="n"/>
+      <c r="T142" s="5" t="n"/>
+      <c r="AT142" s="6" t="n"/>
+      <c r="BJ142" s="6" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="5" t="n"/>
-      <c r="R143" s="5" t="n"/>
+      <c r="B143" s="6" t="n"/>
       <c r="S143" s="6" t="n"/>
-      <c r="AS143" s="5" t="n"/>
-      <c r="BI143" s="5" t="n"/>
+      <c r="T143" s="5" t="n"/>
+      <c r="AT143" s="6" t="n"/>
+      <c r="BJ143" s="6" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="n"/>
-      <c r="R144" s="5" t="n"/>
+      <c r="B144" s="6" t="n"/>
       <c r="S144" s="6" t="n"/>
-      <c r="AS144" s="5" t="n"/>
-      <c r="BI144" s="5" t="n"/>
+      <c r="T144" s="5" t="n"/>
+      <c r="AT144" s="6" t="n"/>
+      <c r="BJ144" s="6" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="5" t="n"/>
-      <c r="R145" s="5" t="n"/>
+      <c r="B145" s="6" t="n"/>
       <c r="S145" s="6" t="n"/>
-      <c r="AS145" s="5" t="n"/>
-      <c r="BI145" s="5" t="n"/>
+      <c r="T145" s="5" t="n"/>
+      <c r="AT145" s="6" t="n"/>
+      <c r="BJ145" s="6" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="n"/>
-      <c r="R146" s="5" t="n"/>
+      <c r="B146" s="6" t="n"/>
       <c r="S146" s="6" t="n"/>
-      <c r="AS146" s="5" t="n"/>
-      <c r="BI146" s="5" t="n"/>
+      <c r="T146" s="5" t="n"/>
+      <c r="AT146" s="6" t="n"/>
+      <c r="BJ146" s="6" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="5" t="n"/>
-      <c r="R147" s="5" t="n"/>
+      <c r="B147" s="6" t="n"/>
       <c r="S147" s="6" t="n"/>
-      <c r="AS147" s="5" t="n"/>
-      <c r="BI147" s="5" t="n"/>
+      <c r="T147" s="5" t="n"/>
+      <c r="AT147" s="6" t="n"/>
+      <c r="BJ147" s="6" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="5" t="n"/>
-      <c r="R148" s="5" t="n"/>
+      <c r="B148" s="6" t="n"/>
       <c r="S148" s="6" t="n"/>
-      <c r="AS148" s="5" t="n"/>
-      <c r="BI148" s="5" t="n"/>
+      <c r="T148" s="5" t="n"/>
+      <c r="AT148" s="6" t="n"/>
+      <c r="BJ148" s="6" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="5" t="n"/>
-      <c r="R149" s="5" t="n"/>
+      <c r="B149" s="6" t="n"/>
       <c r="S149" s="6" t="n"/>
-      <c r="AS149" s="5" t="n"/>
-      <c r="BI149" s="5" t="n"/>
+      <c r="T149" s="5" t="n"/>
+      <c r="AT149" s="6" t="n"/>
+      <c r="BJ149" s="6" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="5" t="n"/>
-      <c r="R150" s="5" t="n"/>
+      <c r="B150" s="6" t="n"/>
       <c r="S150" s="6" t="n"/>
-      <c r="AS150" s="5" t="n"/>
-      <c r="BI150" s="5" t="n"/>
+      <c r="T150" s="5" t="n"/>
+      <c r="AT150" s="6" t="n"/>
+      <c r="BJ150" s="6" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="5" t="n"/>
-      <c r="R151" s="5" t="n"/>
+      <c r="B151" s="6" t="n"/>
       <c r="S151" s="6" t="n"/>
-      <c r="AS151" s="5" t="n"/>
-      <c r="BI151" s="5" t="n"/>
+      <c r="T151" s="5" t="n"/>
+      <c r="AT151" s="6" t="n"/>
+      <c r="BJ151" s="6" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="5" t="n"/>
-      <c r="R152" s="5" t="n"/>
+      <c r="B152" s="6" t="n"/>
       <c r="S152" s="6" t="n"/>
-      <c r="AS152" s="5" t="n"/>
-      <c r="BI152" s="5" t="n"/>
+      <c r="T152" s="5" t="n"/>
+      <c r="AT152" s="6" t="n"/>
+      <c r="BJ152" s="6" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="5" t="n"/>
-      <c r="R153" s="5" t="n"/>
+      <c r="B153" s="6" t="n"/>
       <c r="S153" s="6" t="n"/>
-      <c r="AS153" s="5" t="n"/>
-      <c r="BI153" s="5" t="n"/>
+      <c r="T153" s="5" t="n"/>
+      <c r="AT153" s="6" t="n"/>
+      <c r="BJ153" s="6" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="5" t="n"/>
-      <c r="R154" s="5" t="n"/>
+      <c r="B154" s="6" t="n"/>
       <c r="S154" s="6" t="n"/>
-      <c r="AS154" s="5" t="n"/>
-      <c r="BI154" s="5" t="n"/>
+      <c r="T154" s="5" t="n"/>
+      <c r="AT154" s="6" t="n"/>
+      <c r="BJ154" s="6" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="5" t="n"/>
-      <c r="R155" s="5" t="n"/>
+      <c r="B155" s="6" t="n"/>
       <c r="S155" s="6" t="n"/>
-      <c r="AS155" s="5" t="n"/>
-      <c r="BI155" s="5" t="n"/>
+      <c r="T155" s="5" t="n"/>
+      <c r="AT155" s="6" t="n"/>
+      <c r="BJ155" s="6" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="5" t="n"/>
-      <c r="R156" s="5" t="n"/>
+      <c r="B156" s="6" t="n"/>
       <c r="S156" s="6" t="n"/>
-      <c r="AS156" s="5" t="n"/>
-      <c r="BI156" s="5" t="n"/>
+      <c r="T156" s="5" t="n"/>
+      <c r="AT156" s="6" t="n"/>
+      <c r="BJ156" s="6" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="5" t="n"/>
-      <c r="R157" s="5" t="n"/>
+      <c r="B157" s="6" t="n"/>
       <c r="S157" s="6" t="n"/>
-      <c r="AS157" s="5" t="n"/>
-      <c r="BI157" s="5" t="n"/>
+      <c r="T157" s="5" t="n"/>
+      <c r="AT157" s="6" t="n"/>
+      <c r="BJ157" s="6" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="5" t="n"/>
-      <c r="R158" s="5" t="n"/>
+      <c r="B158" s="6" t="n"/>
       <c r="S158" s="6" t="n"/>
-      <c r="AS158" s="5" t="n"/>
-      <c r="BI158" s="5" t="n"/>
+      <c r="T158" s="5" t="n"/>
+      <c r="AT158" s="6" t="n"/>
+      <c r="BJ158" s="6" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="5" t="n"/>
-      <c r="R159" s="5" t="n"/>
+      <c r="B159" s="6" t="n"/>
       <c r="S159" s="6" t="n"/>
-      <c r="AS159" s="5" t="n"/>
-      <c r="BI159" s="5" t="n"/>
+      <c r="T159" s="5" t="n"/>
+      <c r="AT159" s="6" t="n"/>
+      <c r="BJ159" s="6" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="5" t="n"/>
-      <c r="R160" s="5" t="n"/>
+      <c r="B160" s="6" t="n"/>
       <c r="S160" s="6" t="n"/>
-      <c r="AS160" s="5" t="n"/>
-      <c r="BI160" s="5" t="n"/>
+      <c r="T160" s="5" t="n"/>
+      <c r="AT160" s="6" t="n"/>
+      <c r="BJ160" s="6" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="5" t="n"/>
-      <c r="R161" s="5" t="n"/>
+      <c r="B161" s="6" t="n"/>
       <c r="S161" s="6" t="n"/>
-      <c r="AS161" s="5" t="n"/>
-      <c r="BI161" s="5" t="n"/>
+      <c r="T161" s="5" t="n"/>
+      <c r="AT161" s="6" t="n"/>
+      <c r="BJ161" s="6" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="5" t="n"/>
-      <c r="R162" s="5" t="n"/>
+      <c r="B162" s="6" t="n"/>
       <c r="S162" s="6" t="n"/>
-      <c r="AS162" s="5" t="n"/>
-      <c r="BI162" s="5" t="n"/>
+      <c r="T162" s="5" t="n"/>
+      <c r="AT162" s="6" t="n"/>
+      <c r="BJ162" s="6" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="5" t="n"/>
-      <c r="R163" s="5" t="n"/>
+      <c r="B163" s="6" t="n"/>
       <c r="S163" s="6" t="n"/>
-      <c r="AS163" s="5" t="n"/>
-      <c r="BI163" s="5" t="n"/>
+      <c r="T163" s="5" t="n"/>
+      <c r="AT163" s="6" t="n"/>
+      <c r="BJ163" s="6" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="5" t="n"/>
-      <c r="R164" s="5" t="n"/>
+      <c r="B164" s="6" t="n"/>
       <c r="S164" s="6" t="n"/>
-      <c r="AS164" s="5" t="n"/>
-      <c r="BI164" s="5" t="n"/>
+      <c r="T164" s="5" t="n"/>
+      <c r="AT164" s="6" t="n"/>
+      <c r="BJ164" s="6" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="5" t="n"/>
-      <c r="R165" s="5" t="n"/>
+      <c r="B165" s="6" t="n"/>
       <c r="S165" s="6" t="n"/>
-      <c r="AS165" s="5" t="n"/>
-      <c r="BI165" s="5" t="n"/>
+      <c r="T165" s="5" t="n"/>
+      <c r="AT165" s="6" t="n"/>
+      <c r="BJ165" s="6" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="5" t="n"/>
-      <c r="R166" s="5" t="n"/>
+      <c r="B166" s="6" t="n"/>
       <c r="S166" s="6" t="n"/>
-      <c r="AS166" s="5" t="n"/>
-      <c r="BI166" s="5" t="n"/>
+      <c r="T166" s="5" t="n"/>
+      <c r="AT166" s="6" t="n"/>
+      <c r="BJ166" s="6" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="5" t="n"/>
-      <c r="R167" s="5" t="n"/>
+      <c r="B167" s="6" t="n"/>
       <c r="S167" s="6" t="n"/>
-      <c r="AS167" s="5" t="n"/>
-      <c r="BI167" s="5" t="n"/>
+      <c r="T167" s="5" t="n"/>
+      <c r="AT167" s="6" t="n"/>
+      <c r="BJ167" s="6" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="5" t="n"/>
-      <c r="R168" s="5" t="n"/>
+      <c r="B168" s="6" t="n"/>
       <c r="S168" s="6" t="n"/>
-      <c r="AS168" s="5" t="n"/>
-      <c r="BI168" s="5" t="n"/>
+      <c r="T168" s="5" t="n"/>
+      <c r="AT168" s="6" t="n"/>
+      <c r="BJ168" s="6" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="5" t="n"/>
-      <c r="R169" s="5" t="n"/>
+      <c r="B169" s="6" t="n"/>
       <c r="S169" s="6" t="n"/>
-      <c r="AS169" s="5" t="n"/>
-      <c r="BI169" s="5" t="n"/>
+      <c r="T169" s="5" t="n"/>
+      <c r="AT169" s="6" t="n"/>
+      <c r="BJ169" s="6" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="5" t="n"/>
-      <c r="R170" s="5" t="n"/>
+      <c r="B170" s="6" t="n"/>
       <c r="S170" s="6" t="n"/>
-      <c r="AS170" s="5" t="n"/>
-      <c r="BI170" s="5" t="n"/>
+      <c r="T170" s="5" t="n"/>
+      <c r="AT170" s="6" t="n"/>
+      <c r="BJ170" s="6" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="5" t="n"/>
-      <c r="R171" s="5" t="n"/>
+      <c r="B171" s="6" t="n"/>
       <c r="S171" s="6" t="n"/>
-      <c r="AS171" s="5" t="n"/>
-      <c r="BI171" s="5" t="n"/>
+      <c r="T171" s="5" t="n"/>
+      <c r="AT171" s="6" t="n"/>
+      <c r="BJ171" s="6" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="5" t="n"/>
-      <c r="R172" s="5" t="n"/>
+      <c r="B172" s="6" t="n"/>
       <c r="S172" s="6" t="n"/>
-      <c r="AS172" s="5" t="n"/>
-      <c r="BI172" s="5" t="n"/>
+      <c r="T172" s="5" t="n"/>
+      <c r="AT172" s="6" t="n"/>
+      <c r="BJ172" s="6" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="5" t="n"/>
-      <c r="R173" s="5" t="n"/>
+      <c r="B173" s="6" t="n"/>
       <c r="S173" s="6" t="n"/>
-      <c r="AS173" s="5" t="n"/>
-      <c r="BI173" s="5" t="n"/>
+      <c r="T173" s="5" t="n"/>
+      <c r="AT173" s="6" t="n"/>
+      <c r="BJ173" s="6" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="5" t="n"/>
-      <c r="R174" s="5" t="n"/>
+      <c r="B174" s="6" t="n"/>
       <c r="S174" s="6" t="n"/>
-      <c r="AS174" s="5" t="n"/>
-      <c r="BI174" s="5" t="n"/>
+      <c r="T174" s="5" t="n"/>
+      <c r="AT174" s="6" t="n"/>
+      <c r="BJ174" s="6" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="5" t="n"/>
-      <c r="R175" s="5" t="n"/>
+      <c r="B175" s="6" t="n"/>
       <c r="S175" s="6" t="n"/>
-      <c r="AS175" s="5" t="n"/>
-      <c r="BI175" s="5" t="n"/>
+      <c r="T175" s="5" t="n"/>
+      <c r="AT175" s="6" t="n"/>
+      <c r="BJ175" s="6" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="5" t="n"/>
-      <c r="R176" s="5" t="n"/>
+      <c r="B176" s="6" t="n"/>
       <c r="S176" s="6" t="n"/>
-      <c r="AS176" s="5" t="n"/>
-      <c r="BI176" s="5" t="n"/>
+      <c r="T176" s="5" t="n"/>
+      <c r="AT176" s="6" t="n"/>
+      <c r="BJ176" s="6" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="5" t="n"/>
-      <c r="R177" s="5" t="n"/>
+      <c r="B177" s="6" t="n"/>
       <c r="S177" s="6" t="n"/>
-      <c r="AS177" s="5" t="n"/>
-      <c r="BI177" s="5" t="n"/>
+      <c r="T177" s="5" t="n"/>
+      <c r="AT177" s="6" t="n"/>
+      <c r="BJ177" s="6" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="5" t="n"/>
-      <c r="R178" s="5" t="n"/>
+      <c r="B178" s="6" t="n"/>
       <c r="S178" s="6" t="n"/>
-      <c r="AS178" s="5" t="n"/>
-      <c r="BI178" s="5" t="n"/>
+      <c r="T178" s="5" t="n"/>
+      <c r="AT178" s="6" t="n"/>
+      <c r="BJ178" s="6" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="5" t="n"/>
-      <c r="R179" s="5" t="n"/>
+      <c r="B179" s="6" t="n"/>
       <c r="S179" s="6" t="n"/>
-      <c r="AS179" s="5" t="n"/>
-      <c r="BI179" s="5" t="n"/>
+      <c r="T179" s="5" t="n"/>
+      <c r="AT179" s="6" t="n"/>
+      <c r="BJ179" s="6" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="5" t="n"/>
-      <c r="R180" s="5" t="n"/>
+      <c r="B180" s="6" t="n"/>
       <c r="S180" s="6" t="n"/>
-      <c r="AS180" s="5" t="n"/>
-      <c r="BI180" s="5" t="n"/>
+      <c r="T180" s="5" t="n"/>
+      <c r="AT180" s="6" t="n"/>
+      <c r="BJ180" s="6" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="5" t="n"/>
-      <c r="R181" s="5" t="n"/>
+      <c r="B181" s="6" t="n"/>
       <c r="S181" s="6" t="n"/>
-      <c r="AS181" s="5" t="n"/>
-      <c r="BI181" s="5" t="n"/>
+      <c r="T181" s="5" t="n"/>
+      <c r="AT181" s="6" t="n"/>
+      <c r="BJ181" s="6" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="5" t="n"/>
-      <c r="R182" s="5" t="n"/>
+      <c r="B182" s="6" t="n"/>
       <c r="S182" s="6" t="n"/>
-      <c r="AS182" s="5" t="n"/>
-      <c r="BI182" s="5" t="n"/>
+      <c r="T182" s="5" t="n"/>
+      <c r="AT182" s="6" t="n"/>
+      <c r="BJ182" s="6" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="5" t="n"/>
-      <c r="R183" s="5" t="n"/>
+      <c r="B183" s="6" t="n"/>
       <c r="S183" s="6" t="n"/>
-      <c r="AS183" s="5" t="n"/>
-      <c r="BI183" s="5" t="n"/>
+      <c r="T183" s="5" t="n"/>
+      <c r="AT183" s="6" t="n"/>
+      <c r="BJ183" s="6" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="5" t="n"/>
-      <c r="R184" s="5" t="n"/>
+      <c r="B184" s="6" t="n"/>
       <c r="S184" s="6" t="n"/>
-      <c r="AS184" s="5" t="n"/>
-      <c r="BI184" s="5" t="n"/>
+      <c r="T184" s="5" t="n"/>
+      <c r="AT184" s="6" t="n"/>
+      <c r="BJ184" s="6" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="5" t="n"/>
-      <c r="R185" s="5" t="n"/>
+      <c r="B185" s="6" t="n"/>
       <c r="S185" s="6" t="n"/>
-      <c r="AS185" s="5" t="n"/>
-      <c r="BI185" s="5" t="n"/>
+      <c r="T185" s="5" t="n"/>
+      <c r="AT185" s="6" t="n"/>
+      <c r="BJ185" s="6" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="5" t="n"/>
-      <c r="R186" s="5" t="n"/>
+      <c r="B186" s="6" t="n"/>
       <c r="S186" s="6" t="n"/>
-      <c r="AS186" s="5" t="n"/>
-      <c r="BI186" s="5" t="n"/>
+      <c r="T186" s="5" t="n"/>
+      <c r="AT186" s="6" t="n"/>
+      <c r="BJ186" s="6" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="5" t="n"/>
-      <c r="R187" s="5" t="n"/>
+      <c r="B187" s="6" t="n"/>
       <c r="S187" s="6" t="n"/>
-      <c r="AS187" s="5" t="n"/>
-      <c r="BI187" s="5" t="n"/>
+      <c r="T187" s="5" t="n"/>
+      <c r="AT187" s="6" t="n"/>
+      <c r="BJ187" s="6" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="5" t="n"/>
-      <c r="R188" s="5" t="n"/>
+      <c r="B188" s="6" t="n"/>
       <c r="S188" s="6" t="n"/>
-      <c r="AS188" s="5" t="n"/>
-      <c r="BI188" s="5" t="n"/>
+      <c r="T188" s="5" t="n"/>
+      <c r="AT188" s="6" t="n"/>
+      <c r="BJ188" s="6" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="5" t="n"/>
-      <c r="R189" s="5" t="n"/>
+      <c r="B189" s="6" t="n"/>
       <c r="S189" s="6" t="n"/>
-      <c r="AS189" s="5" t="n"/>
-      <c r="BI189" s="5" t="n"/>
+      <c r="T189" s="5" t="n"/>
+      <c r="AT189" s="6" t="n"/>
+      <c r="BJ189" s="6" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="5" t="n"/>
-      <c r="R190" s="5" t="n"/>
+      <c r="B190" s="6" t="n"/>
       <c r="S190" s="6" t="n"/>
-      <c r="AS190" s="5" t="n"/>
-      <c r="BI190" s="5" t="n"/>
+      <c r="T190" s="5" t="n"/>
+      <c r="AT190" s="6" t="n"/>
+      <c r="BJ190" s="6" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="5" t="n"/>
-      <c r="R191" s="5" t="n"/>
+      <c r="B191" s="6" t="n"/>
       <c r="S191" s="6" t="n"/>
-      <c r="AS191" s="5" t="n"/>
-      <c r="BI191" s="5" t="n"/>
+      <c r="T191" s="5" t="n"/>
+      <c r="AT191" s="6" t="n"/>
+      <c r="BJ191" s="6" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="5" t="n"/>
-      <c r="R192" s="5" t="n"/>
+      <c r="B192" s="6" t="n"/>
       <c r="S192" s="6" t="n"/>
-      <c r="AS192" s="5" t="n"/>
-      <c r="BI192" s="5" t="n"/>
+      <c r="T192" s="5" t="n"/>
+      <c r="AT192" s="6" t="n"/>
+      <c r="BJ192" s="6" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="5" t="n"/>
-      <c r="R193" s="5" t="n"/>
+      <c r="B193" s="6" t="n"/>
       <c r="S193" s="6" t="n"/>
-      <c r="AS193" s="5" t="n"/>
-      <c r="BI193" s="5" t="n"/>
+      <c r="T193" s="5" t="n"/>
+      <c r="AT193" s="6" t="n"/>
+      <c r="BJ193" s="6" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="5" t="n"/>
-      <c r="R194" s="5" t="n"/>
+      <c r="B194" s="6" t="n"/>
       <c r="S194" s="6" t="n"/>
-      <c r="AS194" s="5" t="n"/>
-      <c r="BI194" s="5" t="n"/>
+      <c r="T194" s="5" t="n"/>
+      <c r="AT194" s="6" t="n"/>
+      <c r="BJ194" s="6" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="5" t="n"/>
-      <c r="R195" s="5" t="n"/>
+      <c r="B195" s="6" t="n"/>
       <c r="S195" s="6" t="n"/>
-      <c r="AS195" s="5" t="n"/>
-      <c r="BI195" s="5" t="n"/>
+      <c r="T195" s="5" t="n"/>
+      <c r="AT195" s="6" t="n"/>
+      <c r="BJ195" s="6" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="5" t="n"/>
-      <c r="R196" s="5" t="n"/>
+      <c r="B196" s="6" t="n"/>
       <c r="S196" s="6" t="n"/>
-      <c r="AS196" s="5" t="n"/>
-      <c r="BI196" s="5" t="n"/>
+      <c r="T196" s="5" t="n"/>
+      <c r="AT196" s="6" t="n"/>
+      <c r="BJ196" s="6" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="5" t="n"/>
-      <c r="R197" s="5" t="n"/>
+      <c r="B197" s="6" t="n"/>
       <c r="S197" s="6" t="n"/>
-      <c r="AS197" s="5" t="n"/>
-      <c r="BI197" s="5" t="n"/>
+      <c r="T197" s="5" t="n"/>
+      <c r="AT197" s="6" t="n"/>
+      <c r="BJ197" s="6" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="5" t="n"/>
-      <c r="R198" s="5" t="n"/>
+      <c r="B198" s="6" t="n"/>
       <c r="S198" s="6" t="n"/>
-      <c r="AS198" s="5" t="n"/>
-      <c r="BI198" s="5" t="n"/>
+      <c r="T198" s="5" t="n"/>
+      <c r="AT198" s="6" t="n"/>
+      <c r="BJ198" s="6" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="5" t="n"/>
-      <c r="R199" s="5" t="n"/>
+      <c r="B199" s="6" t="n"/>
       <c r="S199" s="6" t="n"/>
-      <c r="AS199" s="5" t="n"/>
-      <c r="BI199" s="5" t="n"/>
+      <c r="T199" s="5" t="n"/>
+      <c r="AT199" s="6" t="n"/>
+      <c r="BJ199" s="6" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="5" t="n"/>
-      <c r="R200" s="5" t="n"/>
+      <c r="B200" s="6" t="n"/>
       <c r="S200" s="6" t="n"/>
-      <c r="AS200" s="5" t="n"/>
-      <c r="BI200" s="5" t="n"/>
+      <c r="T200" s="5" t="n"/>
+      <c r="AT200" s="6" t="n"/>
+      <c r="BJ200" s="6" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="5" t="n"/>
-      <c r="R201" s="5" t="n"/>
+      <c r="B201" s="6" t="n"/>
       <c r="S201" s="6" t="n"/>
-      <c r="AS201" s="5" t="n"/>
-      <c r="BI201" s="5" t="n"/>
+      <c r="T201" s="5" t="n"/>
+      <c r="AT201" s="6" t="n"/>
+      <c r="BJ201" s="6" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="5" t="n"/>
-      <c r="R202" s="5" t="n"/>
+      <c r="B202" s="6" t="n"/>
       <c r="S202" s="6" t="n"/>
-      <c r="AS202" s="5" t="n"/>
-      <c r="BI202" s="5" t="n"/>
+      <c r="T202" s="5" t="n"/>
+      <c r="AT202" s="6" t="n"/>
+      <c r="BJ202" s="6" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="5" t="n"/>
-      <c r="R203" s="5" t="n"/>
+      <c r="B203" s="6" t="n"/>
       <c r="S203" s="6" t="n"/>
-      <c r="AS203" s="5" t="n"/>
-      <c r="BI203" s="5" t="n"/>
+      <c r="T203" s="5" t="n"/>
+      <c r="AT203" s="6" t="n"/>
+      <c r="BJ203" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="K2:AM2"/>
-    <mergeCell ref="BF2:BK2"/>
-    <mergeCell ref="A1:BL1"/>
-    <mergeCell ref="AN2:BE2"/>
-    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="A1:BM1"/>
+    <mergeCell ref="C2:K2"/>
+    <mergeCell ref="AO2:BF2"/>
+    <mergeCell ref="BG2:BL2"/>
+    <mergeCell ref="L2:AN2"/>
   </mergeCells>
   <dataValidations count="24">
-    <dataValidation sqref="B4:B203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Provincia&quot;." type="list">
+    <dataValidation sqref="C4:C203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Provincia&quot;." type="list">
       <formula1>LISTAS!$M$2:$M$26</formula1>
     </dataValidation>
-    <dataValidation sqref="M4:M203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Situación de documentación&quot;." type="list">
+    <dataValidation sqref="N4:N203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Situación de documentación&quot;." type="list">
       <formula1>LISTAS!$P$2:$P$8</formula1>
     </dataValidation>
-    <dataValidation sqref="P4:P203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Género&quot;." type="list">
+    <dataValidation sqref="Q4:Q203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Género&quot;." type="list">
       <formula1>LISTAS!$D$2:$D$4</formula1>
     </dataValidation>
-    <dataValidation sqref="Q4:Q203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;País de nacimiento&quot;." type="list">
+    <dataValidation sqref="R4:R203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;País de nacimiento&quot;." type="list">
       <formula1>LISTAS!$I$2:$I$247</formula1>
     </dataValidation>
-    <dataValidation sqref="T4:T203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Asistencia escolar&quot;." type="list">
+    <dataValidation sqref="U4:U203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Asistencia escolar&quot;." type="list">
       <formula1>LISTAS!$A$2:$A$4</formula1>
     </dataValidation>
-    <dataValidation sqref="U4:U203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Máximo nivel educativo alcanzado&quot;." type="list">
+    <dataValidation sqref="V4:V203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Máximo nivel educativo alcanzado&quot;." type="list">
       <formula1>LISTAS!$F$2:$F$8</formula1>
     </dataValidation>
-    <dataValidation sqref="W4:W203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Provincia (NyA)&quot;." type="list">
+    <dataValidation sqref="X4:X203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Provincia (NyA)&quot;." type="list">
       <formula1>LISTAS!$M$2:$M$26</formula1>
     </dataValidation>
-    <dataValidation sqref="AA4:AA203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Destinatario&quot;." promptTitle="Destinatario" prompt="Consignar la persona, grupo poblacional o sujeto de derecho al que se dirige la intervención, prestación, acción de acompañamiento o medida de protección." type="list">
+    <dataValidation sqref="AB4:AB203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Destinatario&quot;." promptTitle="Destinatario" prompt="Consignar la persona, grupo poblacional o sujeto de derecho al que se dirige la intervención, prestación, acción de acompañamiento o medida de protección." type="list">
       <formula1>LISTAS!$C$2:$C$4</formula1>
     </dataValidation>
-    <dataValidation sqref="AB4:AB203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Línea de acción&quot;." promptTitle="Línea de acción" prompt="Consignar la estrategia, componente programático, modalidad de intervención o eje de trabajo mediante el cual se implementa la acción de protección, promoción, restitución o fortalecimiento de derechos de NyA." type="list">
+    <dataValidation sqref="AC4:AC203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Línea de acción&quot;." promptTitle="Línea de acción" prompt="Consignar la estrategia, componente programático, modalidad de intervención o eje de trabajo mediante el cual se implementa la acción de protección, promoción, restitución o fortalecimiento de derechos de NyA." type="list">
       <formula1>LISTAS!$E$2:$E$4</formula1>
     </dataValidation>
-    <dataValidation sqref="AD4:AD203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Problemática de salud&quot;." promptTitle="Problemática de salud" prompt="Registrar cualquier situación, condición o dificultad vinculada a la salud física, mental o integral del Ny/Oa que requiera atención, seguimiento, tratamiento o articulación con servicios de salud, independientemente de que constituya o no una enfermedad " type="list">
+    <dataValidation sqref="AE4:AE203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Problemática de salud&quot;." promptTitle="Problemática de salud" prompt="Registrar cualquier situación, condición o dificultad vinculada a la salud física, mental o integral del Ny/Oa que requiera atención, seguimiento, tratamiento o articulación con servicios de salud, independientemente de que constituya o no una enfermedad " type="list">
       <formula1>LISTAS!$L$2:$L$5</formula1>
     </dataValidation>
-    <dataValidation sqref="AF4:AF203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;¿Presenta alguna discapacidad?&quot;." type="list">
+    <dataValidation sqref="AG4:AG203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;¿Presenta alguna discapacidad?&quot;." type="list">
       <formula1>LISTAS!$K$2:$K$4</formula1>
     </dataValidation>
-    <dataValidation sqref="AG4:AG203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Tipo de discapacidad&quot;." type="list">
+    <dataValidation sqref="AH4:AH203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Tipo de discapacidad&quot;." type="list">
       <formula1>LISTAS!$R$2:$R$8</formula1>
     </dataValidation>
-    <dataValidation sqref="AH4:AH203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;¿Posee CUD?&quot;." type="list">
+    <dataValidation sqref="AI4:AI203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;¿Posee CUD?&quot;." type="list">
       <formula1>LISTAS!$J$2:$J$5</formula1>
     </dataValidation>
-    <dataValidation sqref="AI4:AI203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Cobertura salud&quot;." type="list">
+    <dataValidation sqref="AJ4:AJ203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Cobertura salud&quot;." type="list">
       <formula1>LISTAS!$B$2:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="AK4:AK203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;¿Se identifica con algún pueblo originario?&quot;." promptTitle="¿Se identifica con algún pueblo " prompt="Identificar la pertenencia a pueblos originarios para contribuir a la producción de información con enfoque de derechos, diversidad cultural e interculturalidad" type="list">
+    <dataValidation sqref="AL4:AL203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;¿Se identifica con algún pueblo originario?&quot;." promptTitle="¿Se identifica con algún pueblo " prompt="Identificar la pertenencia a pueblos originarios para contribuir a la producción de información con enfoque de derechos, diversidad cultural e interculturalidad" type="list">
       <formula1>LISTAS!$O$2:$O$4</formula1>
     </dataValidation>
-    <dataValidation sqref="AM4:AM203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;¿Tiene hijos/as?&quot;." type="list">
+    <dataValidation sqref="AN4:AN203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;¿Tiene hijos/as?&quot;." type="list">
       <formula1>LISTAS!$K$2:$K$4</formula1>
     </dataValidation>
-    <dataValidation sqref="AN4:AN203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Relación vincular del referente&quot;." type="list">
+    <dataValidation sqref="AO4:AO203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Relación vincular del referente&quot;." type="list">
       <formula1>LISTAS!$N$2:$N$8</formula1>
     </dataValidation>
-    <dataValidation sqref="AR4:AR203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Género del referente&quot;." type="list">
+    <dataValidation sqref="AS4:AS203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Género del referente&quot;." type="list">
       <formula1>LISTAS!$D$2:$D$4</formula1>
     </dataValidation>
-    <dataValidation sqref="AT4:AT203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Nacionalidad del referente&quot;." type="list">
+    <dataValidation sqref="AU4:AU203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Nacionalidad del referente&quot;." type="list">
       <formula1>LISTAS!$I$2:$I$247</formula1>
     </dataValidation>
-    <dataValidation sqref="AY4:AY203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Provincia del referente&quot;." type="list">
+    <dataValidation sqref="AZ4:AZ203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Provincia del referente&quot;." type="list">
       <formula1>LISTAS!$M$2:$M$26</formula1>
     </dataValidation>
-    <dataValidation sqref="BA4:BA203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Nivel escolar del referente&quot;." type="list">
+    <dataValidation sqref="BB4:BB203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Nivel escolar del referente&quot;." type="list">
       <formula1>LISTAS!$G$2:$G$13</formula1>
     </dataValidation>
-    <dataValidation sqref="BB4:BB203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Situación laboral del referente&quot;." type="list">
+    <dataValidation sqref="BC4:BC203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Situación laboral del referente&quot;." type="list">
       <formula1>LISTAS!$Q$2:$Q$4</formula1>
     </dataValidation>
-    <dataValidation sqref="BD4:BD203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;¿El referente se identifica con algún pueblo originario?&quot;." type="list">
+    <dataValidation sqref="BE4:BE203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;¿El referente se identifica con algún pueblo originario?&quot;." type="list">
       <formula1>LISTAS!$O$2:$O$4</formula1>
     </dataValidation>
-    <dataValidation sqref="BG4:BG203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Origen de la demanda&quot;." type="list">
+    <dataValidation sqref="BH4:BH203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no admitido" error="El valor no está entre los admitidos para &quot;Origen de la demanda&quot;." type="list">
       <formula1>LISTAS!$H$2:$H$8</formula1>
     </dataValidation>
   </dataValidations>
@@ -2959,7 +3173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B70"/>
+  <dimension ref="A1:B71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2988,10 +3202,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>ID del Niño, niña o Adolescente</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Identificador que le asigna el sistema provincial al niño, niña o adolescente. Es el mismo que figura en el legajo.
+Campo obligatorio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Fecha del relevamiento</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Consignar la fecha en que se rrealiza el registro o actuliza la informacion.
 Campo obligatorio.
@@ -2999,62 +3226,54 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Dispositivo/espacio</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Provincia</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Debe elegirse un valor de la lista "Provincia".</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Provincia</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Debe elegirse un valor de la lista "Provincia".</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Nombre del programa/dispositivo</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Indicar el nombre del dispositivo, hogar, residencia, centro o programa donde se realiza la intervención.
 Campo obligatorio.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Dependencia institucional</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Registrar la denominación oficial completa de la institución responsable, evitando siglas sin aclaración y nombres abreviados. Si el programa depende de más de un organismo, consignar la dependencia principal.</t>
-        </is>
-      </c>
-    </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Localidad</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n"/>
+          <t>Dependencia institucional</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Registrar la denominación oficial completa de la institución responsable, evitando siglas sin aclaración y nombres abreviados. Si el programa depende de más de un organismo, consignar la dependencia principal.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>Localidad</t>
         </is>
       </c>
       <c r="B9" s="9" t="n"/>
@@ -3062,209 +3281,209 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Equipo interviniente</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Nombre del equipo o área interviniente. Profesionales que participan de la intervención (si corresponde). Disciplina o función de los integrantes cuando sea relevante.</t>
-        </is>
-      </c>
+          <t>Domicilio</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Responsable del programa</t>
+          <t>Equipo interviniente</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Nombre y apellido completos. Cargo o función (si corresponde). Persona formalmente designada como responsable del dispositivo o programa</t>
+          <t>Nombre del equipo o área interviniente. Profesionales que participan de la intervención (si corresponde). Disciplina o función de los integrantes cuando sea relevante.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Teléfono de contacto</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="n"/>
+          <t>Responsable del programa</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Nombre y apellido completos. Cargo o función (si corresponde). Persona formalmente designada como responsable del dispositivo o programa</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Teléfono de contacto</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Mail de contacto</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="B14" s="9" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Niño o adolescente</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Apellido/s</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Registrar el o los apellidos completos del niño, niña o adolescente, de acuerdo con la documentación vigente o, en su defecto, según la información proporcionada por la persona responsable o fuente institucional confiable
 Campo obligatorio.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Nombre/s</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Registrar el o los nombres completos del niño, niña o adolescente, de acuerdo con la documentación vigente o, en su defecto, según la información proporcionada por la persona responsable o fuente institucional confiable
 Campo obligatorio.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Situación de documentación</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Debe elegirse un valor de la lista "Situación de documentación".</t>
-        </is>
-      </c>
-    </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nº DNI</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="n"/>
+          <t>Situación de documentación</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Debe elegirse un valor de la lista "Situación de documentación".</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Nº de CUIL</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>Campo obligatorio.</t>
-        </is>
-      </c>
+          <t>Nº DNI</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Género</t>
+          <t>Nº de CUIL</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Debe elegirse un valor de la lista "Género".</t>
+          <t>Campo obligatorio.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>País de nacimiento</t>
+          <t>Género</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Debe elegirse un valor de la lista "País de nacimiento".</t>
+          <t>Debe elegirse un valor de la lista "Género".</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>País de nacimiento</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Debe elegirse un valor de la lista "País de nacimiento".</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Fecha de nacimiento</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Campo obligatorio.
 Formato de fecha: dd/mm/aaaa.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Edad</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="n"/>
-    </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Asistencia escolar</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Debe elegirse un valor de la lista "Asistencia escolar".</t>
-        </is>
-      </c>
+          <t>Edad</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Máximo nivel educativo alcanzado</t>
+          <t>Asistencia escolar</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Debe elegirse un valor de la lista "Máximo nivel educativo alcanzado".</t>
+          <t>Debe elegirse un valor de la lista "Asistencia escolar".</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Domicilio actual</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="n"/>
+          <t>Máximo nivel educativo alcanzado</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Debe elegirse un valor de la lista "Máximo nivel educativo alcanzado".</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Provincia (NyA)</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Debe elegirse un valor de la lista "Provincia".</t>
-        </is>
-      </c>
+          <t>Domicilio actual</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Localidad (NyA)</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="n"/>
+          <t>Provincia (NyA)</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Debe elegirse un valor de la lista "Provincia".</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Partido</t>
+          <t>Localidad (NyA)</t>
         </is>
       </c>
       <c r="B29" s="9" t="n"/>
@@ -3272,7 +3491,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Código postal</t>
+          <t>Partido</t>
         </is>
       </c>
       <c r="B30" s="9" t="n"/>
@@ -3280,194 +3499,190 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>Código postal</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Destinatario</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>Consignar la persona, grupo poblacional o sujeto de derecho al que se dirige la intervención, prestación, acción de acompañamiento o medida de protección.
 Debe elegirse un valor de la lista "Destinatario".</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Línea de acción</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Consignar la estrategia, componente programático, modalidad de intervención o eje de trabajo mediante el cual se implementa la acción de protección, promoción, restitución o fortalecimiento de derechos de NyA.
 Debe elegirse un valor de la lista "Línea de acción".</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Enfermedad crónica</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>Registrar únicamente enfermedades crónicas diagnosticadas o informadas por fuentes confiables</t>
-        </is>
-      </c>
-    </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Enfermedad crónica</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Registrar únicamente enfermedades crónicas diagnosticadas o informadas por fuentes confiables</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Problemática de salud</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Registrar cualquier situación, condición o dificultad vinculada a la salud física, mental o integral del Ny/Oa que requiera atención, seguimiento, tratamiento o articulación con servicios de salud, independientemente de que constituya o no una enfermedad crónica
 Debe elegirse un valor de la lista "Problemática de salud".</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Consumo problemático de sustancias</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>Registrar únicamente información conocida, relevada o informada por fuentes confiables. Cuando exista una situación de consumo, describirla de manera breve y objetiva</t>
-        </is>
-      </c>
-    </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>¿Presenta alguna discapacidad?</t>
+          <t>Consumo problemático de sustancias</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Debe elegirse un valor de la lista "¿Presenta alguna discapacidad?".</t>
+          <t>Registrar únicamente información conocida, relevada o informada por fuentes confiables. Cuando exista una situación de consumo, describirla de manera breve y objetiva</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tipo de discapacidad</t>
+          <t>¿Presenta alguna discapacidad?</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>Debe elegirse un valor de la lista "Tipo de discapacidad".</t>
+          <t>Debe elegirse un valor de la lista "¿Presenta alguna discapacidad?".</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>¿Posee CUD?</t>
+          <t>Tipo de discapacidad</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Debe elegirse un valor de la lista "¿Posee CUD?".</t>
+          <t>Debe elegirse un valor de la lista "Tipo de discapacidad".</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cobertura salud</t>
+          <t>¿Posee CUD?</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>Debe elegirse un valor de la lista "Cobertura salud".</t>
+          <t>Debe elegirse un valor de la lista "¿Posee CUD?".</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Seguridad social</t>
+          <t>Cobertura salud</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Registrar todos los beneficios vigentes. Ej:Asignación Universal por Hijo (AUH). Asignación Familiar. Pensión por discapacidad. Pensión no contributiva. Programa de acompañamiento social. Otro beneficio social</t>
+          <t>Debe elegirse un valor de la lista "Cobertura salud".</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>Seguridad social</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Registrar todos los beneficios vigentes. Ej:Asignación Universal por Hijo (AUH). Asignación Familiar. Pensión por discapacidad. Pensión no contributiva. Programa de acompañamiento social. Otro beneficio social</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>¿Se identifica con algún pueblo originario?</t>
         </is>
       </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="B42" s="9" t="inlineStr">
         <is>
           <t>Identificar la pertenencia a pueblos originarios para contribuir a la producción de información con enfoque de derechos, diversidad cultural e interculturalidad
 Debe elegirse un valor de la lista "Sí / No / Sin datos".</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Pueblo originario (especificar)</t>
-        </is>
-      </c>
-      <c r="B42" s="9" t="n"/>
-    </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>Pueblo originario (especificar)</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>¿Tiene hijos/as?</t>
         </is>
       </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>Debe elegirse un valor de la lista "¿Presenta alguna discapacidad?".</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>Referente</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Relación vincular del referente</t>
-        </is>
-      </c>
-      <c r="B45" s="9" t="inlineStr">
-        <is>
-          <t>Debe elegirse un valor de la lista "Relación vincular del referente".</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Apellido/s del referente</t>
+          <t>Relación vincular del referente</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>Campo obligatorio.</t>
+          <t>Debe elegirse un valor de la lista "Relación vincular del referente".</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Nombre/s del referente</t>
+          <t>Apellido/s del referente</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
@@ -3479,7 +3694,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DNI del referente</t>
+          <t>Nombre/s del referente</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
@@ -3491,52 +3706,56 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Género del referente</t>
+          <t>DNI del referente</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>Debe elegirse un valor de la lista "Género".</t>
+          <t>Campo obligatorio.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>Género del referente</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>Debe elegirse un valor de la lista "Género".</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>Fecha de nacimiento del referente</t>
         </is>
       </c>
-      <c r="B50" s="9" t="inlineStr">
+      <c r="B51" s="9" t="inlineStr">
         <is>
           <t>Campo obligatorio.
 Formato de fecha: dd/mm/aaaa.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Nacionalidad del referente</t>
-        </is>
-      </c>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>Debe elegirse un valor de la lista "País de nacimiento".</t>
-        </is>
-      </c>
-    </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Domicilio actual del referente</t>
-        </is>
-      </c>
-      <c r="B52" s="9" t="n"/>
+          <t>Nacionalidad del referente</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>Debe elegirse un valor de la lista "País de nacimiento".</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Código postal del referente</t>
+          <t>Domicilio actual del referente</t>
         </is>
       </c>
       <c r="B53" s="9" t="n"/>
@@ -3544,7 +3763,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Localidad del referente</t>
+          <t>Código postal del referente</t>
         </is>
       </c>
       <c r="B54" s="9" t="n"/>
@@ -3552,7 +3771,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Partido del referente</t>
+          <t>Localidad del referente</t>
         </is>
       </c>
       <c r="B55" s="9" t="n"/>
@@ -3560,162 +3779,170 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Provincia del referente</t>
-        </is>
-      </c>
-      <c r="B56" s="9" t="inlineStr">
-        <is>
-          <t>Debe elegirse un valor de la lista "Provincia".</t>
-        </is>
-      </c>
+          <t>Partido del referente</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Teléfono y mail del referente</t>
-        </is>
-      </c>
-      <c r="B57" s="9" t="n"/>
+          <t>Provincia del referente</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>Debe elegirse un valor de la lista "Provincia".</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Nivel escolar del referente</t>
-        </is>
-      </c>
-      <c r="B58" s="9" t="inlineStr">
-        <is>
-          <t>Debe elegirse un valor de la lista "Máximo nivel educativo alcanzado".</t>
-        </is>
-      </c>
+          <t>Teléfono y mail del referente</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="n"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Situación laboral del referente</t>
+          <t>Nivel escolar del referente</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>Debe elegirse un valor de la lista "Situación laboral del referente".</t>
+          <t>Debe elegirse un valor de la lista "Máximo nivel educativo alcanzado".</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Seguridad social del referente</t>
-        </is>
-      </c>
-      <c r="B60" s="9" t="n"/>
+          <t>Situación laboral del referente</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>Debe elegirse un valor de la lista "Situación laboral del referente".</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>¿El referente se identifica con algún pueblo originario?</t>
-        </is>
-      </c>
-      <c r="B61" s="9" t="inlineStr">
-        <is>
-          <t>Debe elegirse un valor de la lista "Sí / No / Sin datos".</t>
-        </is>
-      </c>
+          <t>Seguridad social del referente</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="n"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>¿El referente se identifica con algún pueblo originario?</t>
+        </is>
+      </c>
+      <c r="B62" s="9" t="inlineStr">
+        <is>
+          <t>Debe elegirse un valor de la lista "Sí / No / Sin datos".</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>Pueblo originario del refrente</t>
         </is>
       </c>
-      <c r="B62" s="9" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="10" t="inlineStr">
+      <c r="B63" s="9" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="inlineStr">
         <is>
           <t>Medida</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Equipo Interviniente</t>
-        </is>
-      </c>
-      <c r="B64" s="9" t="inlineStr">
-        <is>
-          <t>Debe identificarse prioritariamente el equipo, área o servicio de pertenencia. Si intervienen varios equipos, consignar el que tenga la responsabilidad principal de la medida o coordinación del caso.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Origen de la demanda</t>
+          <t>Equipo Interviniente</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
         <is>
-          <t>Debe elegirse un valor de la lista "Origen de la demanda".</t>
+          <t>Debe identificarse prioritariamente el equipo, área o servicio de pertenencia. Si intervienen varios equipos, consignar el que tenga la responsabilidad principal de la medida o coordinación del caso.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Causas de las medidas</t>
+          <t>Origen de la demanda</t>
         </is>
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>Mencionar la causa principal que motivó la implementación de la medida. Cuando existan múltiples situaciones de vulneración, registrar aquella que resulte predominante o que haya dado origen a la intervención.</t>
+          <t>Debe elegirse un valor de la lista "Origen de la demanda".</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
+          <t>Causas de las medidas</t>
+        </is>
+      </c>
+      <c r="B67" s="9" t="inlineStr">
+        <is>
+          <t>Mencionar la causa principal que motivó la implementación de la medida. Cuando existan múltiples situaciones de vulneración, registrar aquella que resulte predominante o que haya dado origen a la intervención.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>Fecha de la medida MPI</t>
         </is>
       </c>
-      <c r="B67" s="9" t="inlineStr">
+      <c r="B68" s="9" t="inlineStr">
         <is>
           <t>Registrar la fecha en que se dictó, dispuso o formalizó la Medida de Protección Integral (MPI) por parte de la autoridad administrativa competente. Esta fecha marca el inicio formal de la intervención en el marco de la medida
 Formato de fecha: dd/mm/aaaa.</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Plazos en la intervención</t>
-        </is>
-      </c>
-      <c r="B68" s="9" t="inlineStr">
-        <is>
-          <t>Consignar el período previsto o establecido para la implementación, seguimiento y evaluación de la Medida de Protección Integral (MPI), de acuerdo con la planificación realizada por el organismo o equipo interviniente.</t>
-        </is>
-      </c>
-    </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Causas del cese de la MPI</t>
+          <t>Plazos en la intervención</t>
         </is>
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>Identificar los motivos de finalización de las Medidas de Protección Integral y contribuir al monitoreo de los resultados alcanzados en los procesos de restitución y garantía de derechos</t>
+          <t>Consignar el período previsto o establecido para la implementación, seguimiento y evaluación de la Medida de Protección Integral (MPI), de acuerdo con la planificación realizada por el organismo o equipo interviniente.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
+          <t>Causas del cese de la MPI</t>
+        </is>
+      </c>
+      <c r="B70" s="9" t="inlineStr">
+        <is>
+          <t>Identificar los motivos de finalización de las Medidas de Protección Integral y contribuir al monitoreo de los resultados alcanzados en los procesos de restitución y garantía de derechos</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="B70" s="9" t="inlineStr">
+      <c r="B71" s="9" t="inlineStr">
         <is>
           <t>Registrar información complementaria relevante que contribuya a una mejor comprensión de la situación del niño, niña o adolescente, de su contexto familiar o de la intervención realizada, y que no haya sido consignada en otros campos del formulario.</t>
         </is>

</xml_diff>